<commit_message>
coa mapping and prompt changes
</commit_message>
<xml_diff>
--- a/parquet - schema/CoaDetails.xlsx
+++ b/parquet - schema/CoaDetails.xlsx
@@ -510,10 +510,6 @@
       <c r="H2" t="n">
         <v>1</v>
       </c>
-      <c r="I2" t="inlineStr"/>
-      <c r="J2" t="inlineStr"/>
-      <c r="K2" t="inlineStr"/>
-      <c r="L2" t="inlineStr"/>
       <c r="M2" t="n">
         <v>1</v>
       </c>
@@ -545,10 +541,6 @@
       <c r="H3" t="n">
         <v>2</v>
       </c>
-      <c r="I3" t="inlineStr"/>
-      <c r="J3" t="inlineStr"/>
-      <c r="K3" t="inlineStr"/>
-      <c r="L3" t="inlineStr"/>
       <c r="M3" t="n">
         <v>1</v>
       </c>
@@ -580,10 +572,6 @@
       <c r="H4" t="n">
         <v>2</v>
       </c>
-      <c r="I4" t="inlineStr"/>
-      <c r="J4" t="inlineStr"/>
-      <c r="K4" t="inlineStr"/>
-      <c r="L4" t="inlineStr"/>
       <c r="M4" t="n">
         <v>1</v>
       </c>
@@ -615,10 +603,6 @@
       <c r="H5" t="n">
         <v>2</v>
       </c>
-      <c r="I5" t="inlineStr"/>
-      <c r="J5" t="inlineStr"/>
-      <c r="K5" t="inlineStr"/>
-      <c r="L5" t="inlineStr"/>
       <c r="M5" t="n">
         <v>1</v>
       </c>
@@ -650,10 +634,6 @@
       <c r="H6" t="n">
         <v>2</v>
       </c>
-      <c r="I6" t="inlineStr"/>
-      <c r="J6" t="inlineStr"/>
-      <c r="K6" t="inlineStr"/>
-      <c r="L6" t="inlineStr"/>
       <c r="M6" t="n">
         <v>1</v>
       </c>
@@ -685,10 +665,6 @@
       <c r="H7" t="n">
         <v>2</v>
       </c>
-      <c r="I7" t="inlineStr"/>
-      <c r="J7" t="inlineStr"/>
-      <c r="K7" t="inlineStr"/>
-      <c r="L7" t="inlineStr"/>
       <c r="M7" t="n">
         <v>1</v>
       </c>
@@ -720,10 +696,6 @@
       <c r="H8" t="n">
         <v>2</v>
       </c>
-      <c r="I8" t="inlineStr"/>
-      <c r="J8" t="inlineStr"/>
-      <c r="K8" t="inlineStr"/>
-      <c r="L8" t="inlineStr"/>
       <c r="M8" t="n">
         <v>1</v>
       </c>
@@ -755,10 +727,6 @@
       <c r="H9" t="n">
         <v>2</v>
       </c>
-      <c r="I9" t="inlineStr"/>
-      <c r="J9" t="inlineStr"/>
-      <c r="K9" t="inlineStr"/>
-      <c r="L9" t="inlineStr"/>
       <c r="M9" t="n">
         <v>1</v>
       </c>
@@ -790,10 +758,6 @@
       <c r="H10" t="n">
         <v>2</v>
       </c>
-      <c r="I10" t="inlineStr"/>
-      <c r="J10" t="inlineStr"/>
-      <c r="K10" t="inlineStr"/>
-      <c r="L10" t="inlineStr"/>
       <c r="M10" t="n">
         <v>1</v>
       </c>
@@ -825,10 +789,6 @@
       <c r="H11" t="n">
         <v>2</v>
       </c>
-      <c r="I11" t="inlineStr"/>
-      <c r="J11" t="inlineStr"/>
-      <c r="K11" t="inlineStr"/>
-      <c r="L11" t="inlineStr"/>
       <c r="M11" t="n">
         <v>1</v>
       </c>
@@ -842,7 +802,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Prepaid items</t>
+          <t>Prepaid Items</t>
         </is>
       </c>
       <c r="D12" t="n">
@@ -860,10 +820,6 @@
       <c r="H12" t="n">
         <v>2</v>
       </c>
-      <c r="I12" t="inlineStr"/>
-      <c r="J12" t="inlineStr"/>
-      <c r="K12" t="inlineStr"/>
-      <c r="L12" t="inlineStr"/>
       <c r="M12" t="n">
         <v>1</v>
       </c>
@@ -895,10 +851,6 @@
       <c r="H13" t="n">
         <v>2</v>
       </c>
-      <c r="I13" t="inlineStr"/>
-      <c r="J13" t="inlineStr"/>
-      <c r="K13" t="inlineStr"/>
-      <c r="L13" t="inlineStr"/>
       <c r="M13" t="n">
         <v>1</v>
       </c>
@@ -930,10 +882,6 @@
       <c r="H14" t="n">
         <v>2</v>
       </c>
-      <c r="I14" t="inlineStr"/>
-      <c r="J14" t="inlineStr"/>
-      <c r="K14" t="inlineStr"/>
-      <c r="L14" t="inlineStr"/>
       <c r="M14" t="n">
         <v>1</v>
       </c>
@@ -965,10 +913,6 @@
       <c r="H15" t="n">
         <v>2</v>
       </c>
-      <c r="I15" t="inlineStr"/>
-      <c r="J15" t="inlineStr"/>
-      <c r="K15" t="inlineStr"/>
-      <c r="L15" t="inlineStr"/>
       <c r="M15" t="n">
         <v>1</v>
       </c>
@@ -1000,10 +944,6 @@
       <c r="H16" t="n">
         <v>2</v>
       </c>
-      <c r="I16" t="inlineStr"/>
-      <c r="J16" t="inlineStr"/>
-      <c r="K16" t="inlineStr"/>
-      <c r="L16" t="inlineStr"/>
       <c r="M16" t="n">
         <v>1</v>
       </c>
@@ -1035,10 +975,6 @@
       <c r="H17" t="n">
         <v>2</v>
       </c>
-      <c r="I17" t="inlineStr"/>
-      <c r="J17" t="inlineStr"/>
-      <c r="K17" t="inlineStr"/>
-      <c r="L17" t="inlineStr"/>
       <c r="M17" t="n">
         <v>1</v>
       </c>
@@ -1070,10 +1006,6 @@
       <c r="H18" t="n">
         <v>2</v>
       </c>
-      <c r="I18" t="inlineStr"/>
-      <c r="J18" t="inlineStr"/>
-      <c r="K18" t="inlineStr"/>
-      <c r="L18" t="inlineStr"/>
       <c r="M18" t="n">
         <v>1</v>
       </c>
@@ -1105,10 +1037,6 @@
       <c r="H19" t="n">
         <v>2</v>
       </c>
-      <c r="I19" t="inlineStr"/>
-      <c r="J19" t="inlineStr"/>
-      <c r="K19" t="inlineStr"/>
-      <c r="L19" t="inlineStr"/>
       <c r="M19" t="n">
         <v>1</v>
       </c>
@@ -1140,10 +1068,6 @@
       <c r="H20" t="n">
         <v>3</v>
       </c>
-      <c r="I20" t="inlineStr"/>
-      <c r="J20" t="inlineStr"/>
-      <c r="K20" t="inlineStr"/>
-      <c r="L20" t="inlineStr"/>
       <c r="M20" t="n">
         <v>1</v>
       </c>
@@ -1175,10 +1099,6 @@
       <c r="H21" t="n">
         <v>3</v>
       </c>
-      <c r="I21" t="inlineStr"/>
-      <c r="J21" t="inlineStr"/>
-      <c r="K21" t="inlineStr"/>
-      <c r="L21" t="inlineStr"/>
       <c r="M21" t="n">
         <v>1</v>
       </c>
@@ -1210,10 +1130,6 @@
       <c r="H22" t="n">
         <v>3</v>
       </c>
-      <c r="I22" t="inlineStr"/>
-      <c r="J22" t="inlineStr"/>
-      <c r="K22" t="inlineStr"/>
-      <c r="L22" t="inlineStr"/>
       <c r="M22" t="n">
         <v>1</v>
       </c>
@@ -1245,10 +1161,6 @@
       <c r="H23" t="n">
         <v>3</v>
       </c>
-      <c r="I23" t="inlineStr"/>
-      <c r="J23" t="inlineStr"/>
-      <c r="K23" t="inlineStr"/>
-      <c r="L23" t="inlineStr"/>
       <c r="M23" t="n">
         <v>1</v>
       </c>
@@ -1280,10 +1192,6 @@
       <c r="H24" t="n">
         <v>3</v>
       </c>
-      <c r="I24" t="inlineStr"/>
-      <c r="J24" t="inlineStr"/>
-      <c r="K24" t="inlineStr"/>
-      <c r="L24" t="inlineStr"/>
       <c r="M24" t="n">
         <v>1</v>
       </c>
@@ -1315,10 +1223,6 @@
       <c r="H25" t="n">
         <v>3</v>
       </c>
-      <c r="I25" t="inlineStr"/>
-      <c r="J25" t="inlineStr"/>
-      <c r="K25" t="inlineStr"/>
-      <c r="L25" t="inlineStr"/>
       <c r="M25" t="n">
         <v>1</v>
       </c>
@@ -1350,10 +1254,6 @@
       <c r="H26" t="n">
         <v>3</v>
       </c>
-      <c r="I26" t="inlineStr"/>
-      <c r="J26" t="inlineStr"/>
-      <c r="K26" t="inlineStr"/>
-      <c r="L26" t="inlineStr"/>
       <c r="M26" t="n">
         <v>1</v>
       </c>
@@ -1385,10 +1285,6 @@
       <c r="H27" t="n">
         <v>3</v>
       </c>
-      <c r="I27" t="inlineStr"/>
-      <c r="J27" t="inlineStr"/>
-      <c r="K27" t="inlineStr"/>
-      <c r="L27" t="inlineStr"/>
       <c r="M27" t="n">
         <v>1</v>
       </c>
@@ -1420,10 +1316,6 @@
       <c r="H28" t="n">
         <v>1</v>
       </c>
-      <c r="I28" t="inlineStr"/>
-      <c r="J28" t="inlineStr"/>
-      <c r="K28" t="inlineStr"/>
-      <c r="L28" t="inlineStr"/>
       <c r="M28" t="n">
         <v>1</v>
       </c>
@@ -1455,10 +1347,6 @@
       <c r="H29" t="n">
         <v>2</v>
       </c>
-      <c r="I29" t="inlineStr"/>
-      <c r="J29" t="inlineStr"/>
-      <c r="K29" t="inlineStr"/>
-      <c r="L29" t="inlineStr"/>
       <c r="M29" t="n">
         <v>1</v>
       </c>
@@ -1490,10 +1378,6 @@
       <c r="H30" t="n">
         <v>3</v>
       </c>
-      <c r="I30" t="inlineStr"/>
-      <c r="J30" t="inlineStr"/>
-      <c r="K30" t="inlineStr"/>
-      <c r="L30" t="inlineStr"/>
       <c r="M30" t="n">
         <v>1</v>
       </c>
@@ -1525,10 +1409,6 @@
       <c r="H31" t="n">
         <v>3</v>
       </c>
-      <c r="I31" t="inlineStr"/>
-      <c r="J31" t="inlineStr"/>
-      <c r="K31" t="inlineStr"/>
-      <c r="L31" t="inlineStr"/>
       <c r="M31" t="n">
         <v>1</v>
       </c>
@@ -1560,10 +1440,6 @@
       <c r="H32" t="n">
         <v>1</v>
       </c>
-      <c r="I32" t="inlineStr"/>
-      <c r="J32" t="inlineStr"/>
-      <c r="K32" t="inlineStr"/>
-      <c r="L32" t="inlineStr"/>
       <c r="M32" t="n">
         <v>1</v>
       </c>
@@ -1595,10 +1471,6 @@
       <c r="H33" t="n">
         <v>2</v>
       </c>
-      <c r="I33" t="inlineStr"/>
-      <c r="J33" t="inlineStr"/>
-      <c r="K33" t="inlineStr"/>
-      <c r="L33" t="inlineStr"/>
       <c r="M33" t="n">
         <v>1</v>
       </c>
@@ -1630,10 +1502,6 @@
       <c r="H34" t="n">
         <v>2</v>
       </c>
-      <c r="I34" t="inlineStr"/>
-      <c r="J34" t="inlineStr"/>
-      <c r="K34" t="inlineStr"/>
-      <c r="L34" t="inlineStr"/>
       <c r="M34" t="n">
         <v>1</v>
       </c>
@@ -1665,10 +1533,6 @@
       <c r="H35" t="n">
         <v>2</v>
       </c>
-      <c r="I35" t="inlineStr"/>
-      <c r="J35" t="inlineStr"/>
-      <c r="K35" t="inlineStr"/>
-      <c r="L35" t="inlineStr"/>
       <c r="M35" t="n">
         <v>1</v>
       </c>
@@ -1700,10 +1564,6 @@
       <c r="H36" t="n">
         <v>2</v>
       </c>
-      <c r="I36" t="inlineStr"/>
-      <c r="J36" t="inlineStr"/>
-      <c r="K36" t="inlineStr"/>
-      <c r="L36" t="inlineStr"/>
       <c r="M36" t="n">
         <v>1</v>
       </c>
@@ -1735,10 +1595,6 @@
       <c r="H37" t="n">
         <v>2</v>
       </c>
-      <c r="I37" t="inlineStr"/>
-      <c r="J37" t="inlineStr"/>
-      <c r="K37" t="inlineStr"/>
-      <c r="L37" t="inlineStr"/>
       <c r="M37" t="n">
         <v>1</v>
       </c>
@@ -1770,10 +1626,6 @@
       <c r="H38" t="n">
         <v>2</v>
       </c>
-      <c r="I38" t="inlineStr"/>
-      <c r="J38" t="inlineStr"/>
-      <c r="K38" t="inlineStr"/>
-      <c r="L38" t="inlineStr"/>
       <c r="M38" t="n">
         <v>1</v>
       </c>
@@ -1805,10 +1657,6 @@
       <c r="H39" t="n">
         <v>2</v>
       </c>
-      <c r="I39" t="inlineStr"/>
-      <c r="J39" t="inlineStr"/>
-      <c r="K39" t="inlineStr"/>
-      <c r="L39" t="inlineStr"/>
       <c r="M39" t="n">
         <v>1</v>
       </c>
@@ -1840,10 +1688,6 @@
       <c r="H40" t="n">
         <v>2</v>
       </c>
-      <c r="I40" t="inlineStr"/>
-      <c r="J40" t="inlineStr"/>
-      <c r="K40" t="inlineStr"/>
-      <c r="L40" t="inlineStr"/>
       <c r="M40" t="n">
         <v>1</v>
       </c>
@@ -1875,10 +1719,6 @@
       <c r="H41" t="n">
         <v>2</v>
       </c>
-      <c r="I41" t="inlineStr"/>
-      <c r="J41" t="inlineStr"/>
-      <c r="K41" t="inlineStr"/>
-      <c r="L41" t="inlineStr"/>
       <c r="M41" t="n">
         <v>1</v>
       </c>
@@ -1910,10 +1750,6 @@
       <c r="H42" t="n">
         <v>2</v>
       </c>
-      <c r="I42" t="inlineStr"/>
-      <c r="J42" t="inlineStr"/>
-      <c r="K42" t="inlineStr"/>
-      <c r="L42" t="inlineStr"/>
       <c r="M42" t="n">
         <v>1</v>
       </c>
@@ -1945,10 +1781,6 @@
       <c r="H43" t="n">
         <v>2</v>
       </c>
-      <c r="I43" t="inlineStr"/>
-      <c r="J43" t="inlineStr"/>
-      <c r="K43" t="inlineStr"/>
-      <c r="L43" t="inlineStr"/>
       <c r="M43" t="n">
         <v>1</v>
       </c>
@@ -1980,10 +1812,6 @@
       <c r="H44" t="n">
         <v>2</v>
       </c>
-      <c r="I44" t="inlineStr"/>
-      <c r="J44" t="inlineStr"/>
-      <c r="K44" t="inlineStr"/>
-      <c r="L44" t="inlineStr"/>
       <c r="M44" t="n">
         <v>1</v>
       </c>
@@ -2015,10 +1843,6 @@
       <c r="H45" t="n">
         <v>2</v>
       </c>
-      <c r="I45" t="inlineStr"/>
-      <c r="J45" t="inlineStr"/>
-      <c r="K45" t="inlineStr"/>
-      <c r="L45" t="inlineStr"/>
       <c r="M45" t="n">
         <v>1</v>
       </c>
@@ -2050,10 +1874,6 @@
       <c r="H46" t="n">
         <v>2</v>
       </c>
-      <c r="I46" t="inlineStr"/>
-      <c r="J46" t="inlineStr"/>
-      <c r="K46" t="inlineStr"/>
-      <c r="L46" t="inlineStr"/>
       <c r="M46" t="n">
         <v>1</v>
       </c>
@@ -2085,10 +1905,6 @@
       <c r="H47" t="n">
         <v>2</v>
       </c>
-      <c r="I47" t="inlineStr"/>
-      <c r="J47" t="inlineStr"/>
-      <c r="K47" t="inlineStr"/>
-      <c r="L47" t="inlineStr"/>
       <c r="M47" t="n">
         <v>1</v>
       </c>
@@ -2120,10 +1936,6 @@
       <c r="H48" t="n">
         <v>2</v>
       </c>
-      <c r="I48" t="inlineStr"/>
-      <c r="J48" t="inlineStr"/>
-      <c r="K48" t="inlineStr"/>
-      <c r="L48" t="inlineStr"/>
       <c r="M48" t="n">
         <v>1</v>
       </c>
@@ -2155,10 +1967,6 @@
       <c r="H49" t="n">
         <v>2</v>
       </c>
-      <c r="I49" t="inlineStr"/>
-      <c r="J49" t="inlineStr"/>
-      <c r="K49" t="inlineStr"/>
-      <c r="L49" t="inlineStr"/>
       <c r="M49" t="n">
         <v>1</v>
       </c>
@@ -2190,10 +1998,6 @@
       <c r="H50" t="n">
         <v>3</v>
       </c>
-      <c r="I50" t="inlineStr"/>
-      <c r="J50" t="inlineStr"/>
-      <c r="K50" t="inlineStr"/>
-      <c r="L50" t="inlineStr"/>
       <c r="M50" t="n">
         <v>1</v>
       </c>
@@ -2225,10 +2029,6 @@
       <c r="H51" t="n">
         <v>3</v>
       </c>
-      <c r="I51" t="inlineStr"/>
-      <c r="J51" t="inlineStr"/>
-      <c r="K51" t="inlineStr"/>
-      <c r="L51" t="inlineStr"/>
       <c r="M51" t="n">
         <v>1</v>
       </c>
@@ -2260,10 +2060,6 @@
       <c r="H52" t="n">
         <v>3</v>
       </c>
-      <c r="I52" t="inlineStr"/>
-      <c r="J52" t="inlineStr"/>
-      <c r="K52" t="inlineStr"/>
-      <c r="L52" t="inlineStr"/>
       <c r="M52" t="n">
         <v>1</v>
       </c>
@@ -2295,10 +2091,6 @@
       <c r="H53" t="n">
         <v>1</v>
       </c>
-      <c r="I53" t="inlineStr"/>
-      <c r="J53" t="inlineStr"/>
-      <c r="K53" t="inlineStr"/>
-      <c r="L53" t="inlineStr"/>
       <c r="M53" t="n">
         <v>1</v>
       </c>
@@ -2330,10 +2122,6 @@
       <c r="H54" t="n">
         <v>2</v>
       </c>
-      <c r="I54" t="inlineStr"/>
-      <c r="J54" t="inlineStr"/>
-      <c r="K54" t="inlineStr"/>
-      <c r="L54" t="inlineStr"/>
       <c r="M54" t="n">
         <v>1</v>
       </c>
@@ -2365,10 +2153,6 @@
       <c r="H55" t="n">
         <v>3</v>
       </c>
-      <c r="I55" t="inlineStr"/>
-      <c r="J55" t="inlineStr"/>
-      <c r="K55" t="inlineStr"/>
-      <c r="L55" t="inlineStr"/>
       <c r="M55" t="n">
         <v>1</v>
       </c>
@@ -2400,10 +2184,6 @@
       <c r="H56" t="n">
         <v>3</v>
       </c>
-      <c r="I56" t="inlineStr"/>
-      <c r="J56" t="inlineStr"/>
-      <c r="K56" t="inlineStr"/>
-      <c r="L56" t="inlineStr"/>
       <c r="M56" t="n">
         <v>1</v>
       </c>
@@ -2435,10 +2215,6 @@
       <c r="H57" t="n">
         <v>1</v>
       </c>
-      <c r="I57" t="inlineStr"/>
-      <c r="J57" t="inlineStr"/>
-      <c r="K57" t="inlineStr"/>
-      <c r="L57" t="inlineStr"/>
       <c r="M57" t="n">
         <v>1</v>
       </c>
@@ -2470,10 +2246,6 @@
       <c r="H58" t="n">
         <v>2</v>
       </c>
-      <c r="I58" t="inlineStr"/>
-      <c r="J58" t="inlineStr"/>
-      <c r="K58" t="inlineStr"/>
-      <c r="L58" t="inlineStr"/>
       <c r="M58" t="n">
         <v>1</v>
       </c>
@@ -2505,10 +2277,6 @@
       <c r="H59" t="n">
         <v>2</v>
       </c>
-      <c r="I59" t="inlineStr"/>
-      <c r="J59" t="inlineStr"/>
-      <c r="K59" t="inlineStr"/>
-      <c r="L59" t="inlineStr"/>
       <c r="M59" t="n">
         <v>1</v>
       </c>
@@ -2540,10 +2308,6 @@
       <c r="H60" t="n">
         <v>2</v>
       </c>
-      <c r="I60" t="inlineStr"/>
-      <c r="J60" t="inlineStr"/>
-      <c r="K60" t="inlineStr"/>
-      <c r="L60" t="inlineStr"/>
       <c r="M60" t="n">
         <v>1</v>
       </c>
@@ -2575,10 +2339,6 @@
       <c r="H61" t="n">
         <v>3</v>
       </c>
-      <c r="I61" t="inlineStr"/>
-      <c r="J61" t="inlineStr"/>
-      <c r="K61" t="inlineStr"/>
-      <c r="L61" t="inlineStr"/>
       <c r="M61" t="n">
         <v>1</v>
       </c>
@@ -2610,10 +2370,6 @@
       <c r="H62" t="n">
         <v>3</v>
       </c>
-      <c r="I62" t="inlineStr"/>
-      <c r="J62" t="inlineStr"/>
-      <c r="K62" t="inlineStr"/>
-      <c r="L62" t="inlineStr"/>
       <c r="M62" t="n">
         <v>1</v>
       </c>
@@ -2645,10 +2401,6 @@
       <c r="H63" t="n">
         <v>3</v>
       </c>
-      <c r="I63" t="inlineStr"/>
-      <c r="J63" t="inlineStr"/>
-      <c r="K63" t="inlineStr"/>
-      <c r="L63" t="inlineStr"/>
       <c r="M63" t="n">
         <v>1</v>
       </c>
@@ -2680,10 +2432,6 @@
       <c r="H64" t="n">
         <v>3</v>
       </c>
-      <c r="I64" t="inlineStr"/>
-      <c r="J64" t="inlineStr"/>
-      <c r="K64" t="inlineStr"/>
-      <c r="L64" t="inlineStr"/>
       <c r="M64" t="n">
         <v>1</v>
       </c>
@@ -2697,7 +2445,7 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>Total Liabilities, Deferred inflows of resources, and Net position</t>
+          <t>Total Liabilities, Deferred Inflows of Resources, and Net Position</t>
         </is>
       </c>
       <c r="D65" t="n">
@@ -2715,10 +2463,6 @@
       <c r="H65" t="n">
         <v>3</v>
       </c>
-      <c r="I65" t="inlineStr"/>
-      <c r="J65" t="inlineStr"/>
-      <c r="K65" t="inlineStr"/>
-      <c r="L65" t="inlineStr"/>
       <c r="M65" t="n">
         <v>1</v>
       </c>
@@ -2750,10 +2494,6 @@
       <c r="H66" t="n">
         <v>1</v>
       </c>
-      <c r="I66" t="inlineStr"/>
-      <c r="J66" t="inlineStr"/>
-      <c r="K66" t="inlineStr"/>
-      <c r="L66" t="inlineStr"/>
       <c r="M66" t="n">
         <v>1</v>
       </c>
@@ -2785,10 +2525,6 @@
       <c r="H67" t="n">
         <v>2</v>
       </c>
-      <c r="I67" t="inlineStr"/>
-      <c r="J67" t="inlineStr"/>
-      <c r="K67" t="inlineStr"/>
-      <c r="L67" t="inlineStr"/>
       <c r="M67" t="n">
         <v>1</v>
       </c>
@@ -2820,10 +2556,6 @@
       <c r="H68" t="n">
         <v>2</v>
       </c>
-      <c r="I68" t="inlineStr"/>
-      <c r="J68" t="inlineStr"/>
-      <c r="K68" t="inlineStr"/>
-      <c r="L68" t="inlineStr"/>
       <c r="M68" t="n">
         <v>1</v>
       </c>
@@ -2855,10 +2587,6 @@
       <c r="H69" t="n">
         <v>2</v>
       </c>
-      <c r="I69" t="inlineStr"/>
-      <c r="J69" t="inlineStr"/>
-      <c r="K69" t="inlineStr"/>
-      <c r="L69" t="inlineStr"/>
       <c r="M69" t="n">
         <v>1</v>
       </c>
@@ -2890,10 +2618,6 @@
       <c r="H70" t="n">
         <v>2</v>
       </c>
-      <c r="I70" t="inlineStr"/>
-      <c r="J70" t="inlineStr"/>
-      <c r="K70" t="inlineStr"/>
-      <c r="L70" t="inlineStr"/>
       <c r="M70" t="n">
         <v>1</v>
       </c>
@@ -2925,10 +2649,6 @@
       <c r="H71" t="n">
         <v>2</v>
       </c>
-      <c r="I71" t="inlineStr"/>
-      <c r="J71" t="inlineStr"/>
-      <c r="K71" t="inlineStr"/>
-      <c r="L71" t="inlineStr"/>
       <c r="M71" t="n">
         <v>1</v>
       </c>
@@ -2960,10 +2680,6 @@
       <c r="H72" t="n">
         <v>3</v>
       </c>
-      <c r="I72" t="inlineStr"/>
-      <c r="J72" t="inlineStr"/>
-      <c r="K72" t="inlineStr"/>
-      <c r="L72" t="inlineStr"/>
       <c r="M72" t="n">
         <v>1</v>
       </c>
@@ -2995,10 +2711,6 @@
       <c r="H73" t="n">
         <v>3</v>
       </c>
-      <c r="I73" t="inlineStr"/>
-      <c r="J73" t="inlineStr"/>
-      <c r="K73" t="inlineStr"/>
-      <c r="L73" t="inlineStr"/>
       <c r="M73" t="n">
         <v>1</v>
       </c>
@@ -3030,10 +2742,6 @@
       <c r="H74" t="n">
         <v>3</v>
       </c>
-      <c r="I74" t="inlineStr"/>
-      <c r="J74" t="inlineStr"/>
-      <c r="K74" t="inlineStr"/>
-      <c r="L74" t="inlineStr"/>
       <c r="M74" t="n">
         <v>1</v>
       </c>
@@ -3065,10 +2773,6 @@
       <c r="H75" t="n">
         <v>1</v>
       </c>
-      <c r="I75" t="inlineStr"/>
-      <c r="J75" t="inlineStr"/>
-      <c r="K75" t="inlineStr"/>
-      <c r="L75" t="inlineStr"/>
       <c r="M75" t="n">
         <v>1</v>
       </c>
@@ -3100,10 +2804,6 @@
       <c r="H76" t="n">
         <v>2</v>
       </c>
-      <c r="I76" t="inlineStr"/>
-      <c r="J76" t="inlineStr"/>
-      <c r="K76" t="inlineStr"/>
-      <c r="L76" t="inlineStr"/>
       <c r="M76" t="n">
         <v>1</v>
       </c>
@@ -3135,10 +2835,6 @@
       <c r="H77" t="n">
         <v>2</v>
       </c>
-      <c r="I77" t="inlineStr"/>
-      <c r="J77" t="inlineStr"/>
-      <c r="K77" t="inlineStr"/>
-      <c r="L77" t="inlineStr"/>
       <c r="M77" t="n">
         <v>1</v>
       </c>
@@ -3170,10 +2866,6 @@
       <c r="H78" t="n">
         <v>2</v>
       </c>
-      <c r="I78" t="inlineStr"/>
-      <c r="J78" t="inlineStr"/>
-      <c r="K78" t="inlineStr"/>
-      <c r="L78" t="inlineStr"/>
       <c r="M78" t="n">
         <v>1</v>
       </c>
@@ -3205,10 +2897,6 @@
       <c r="H79" t="n">
         <v>2</v>
       </c>
-      <c r="I79" t="inlineStr"/>
-      <c r="J79" t="inlineStr"/>
-      <c r="K79" t="inlineStr"/>
-      <c r="L79" t="inlineStr"/>
       <c r="M79" t="n">
         <v>1</v>
       </c>
@@ -3240,10 +2928,6 @@
       <c r="H80" t="n">
         <v>2</v>
       </c>
-      <c r="I80" t="inlineStr"/>
-      <c r="J80" t="inlineStr"/>
-      <c r="K80" t="inlineStr"/>
-      <c r="L80" t="inlineStr"/>
       <c r="M80" t="n">
         <v>1</v>
       </c>
@@ -3275,10 +2959,6 @@
       <c r="H81" t="n">
         <v>2</v>
       </c>
-      <c r="I81" t="inlineStr"/>
-      <c r="J81" t="inlineStr"/>
-      <c r="K81" t="inlineStr"/>
-      <c r="L81" t="inlineStr"/>
       <c r="M81" t="n">
         <v>1</v>
       </c>
@@ -3310,10 +2990,6 @@
       <c r="H82" t="n">
         <v>2</v>
       </c>
-      <c r="I82" t="inlineStr"/>
-      <c r="J82" t="inlineStr"/>
-      <c r="K82" t="inlineStr"/>
-      <c r="L82" t="inlineStr"/>
       <c r="M82" t="n">
         <v>1</v>
       </c>
@@ -3345,10 +3021,6 @@
       <c r="H83" t="n">
         <v>2</v>
       </c>
-      <c r="I83" t="inlineStr"/>
-      <c r="J83" t="inlineStr"/>
-      <c r="K83" t="inlineStr"/>
-      <c r="L83" t="inlineStr"/>
       <c r="M83" t="n">
         <v>1</v>
       </c>
@@ -3380,10 +3052,6 @@
       <c r="H84" t="n">
         <v>2</v>
       </c>
-      <c r="I84" t="inlineStr"/>
-      <c r="J84" t="inlineStr"/>
-      <c r="K84" t="inlineStr"/>
-      <c r="L84" t="inlineStr"/>
       <c r="M84" t="n">
         <v>1</v>
       </c>
@@ -3415,10 +3083,6 @@
       <c r="H85" t="n">
         <v>3</v>
       </c>
-      <c r="I85" t="inlineStr"/>
-      <c r="J85" t="inlineStr"/>
-      <c r="K85" t="inlineStr"/>
-      <c r="L85" t="inlineStr"/>
       <c r="M85" t="n">
         <v>1</v>
       </c>
@@ -3450,10 +3114,6 @@
       <c r="H86" t="n">
         <v>1</v>
       </c>
-      <c r="I86" t="inlineStr"/>
-      <c r="J86" t="inlineStr"/>
-      <c r="K86" t="inlineStr"/>
-      <c r="L86" t="inlineStr"/>
       <c r="M86" t="n">
         <v>1</v>
       </c>
@@ -3485,10 +3145,6 @@
       <c r="H87" t="n">
         <v>2</v>
       </c>
-      <c r="I87" t="inlineStr"/>
-      <c r="J87" t="inlineStr"/>
-      <c r="K87" t="inlineStr"/>
-      <c r="L87" t="inlineStr"/>
       <c r="M87" t="n">
         <v>1</v>
       </c>
@@ -3520,10 +3176,6 @@
       <c r="H88" t="n">
         <v>3</v>
       </c>
-      <c r="I88" t="inlineStr"/>
-      <c r="J88" t="inlineStr"/>
-      <c r="K88" t="inlineStr"/>
-      <c r="L88" t="inlineStr"/>
       <c r="M88" t="n">
         <v>1</v>
       </c>
@@ -3555,10 +3207,6 @@
       <c r="H89" t="n">
         <v>1</v>
       </c>
-      <c r="I89" t="inlineStr"/>
-      <c r="J89" t="inlineStr"/>
-      <c r="K89" t="inlineStr"/>
-      <c r="L89" t="inlineStr"/>
       <c r="M89" t="n">
         <v>1</v>
       </c>
@@ -3590,10 +3238,6 @@
       <c r="H90" t="n">
         <v>2</v>
       </c>
-      <c r="I90" t="inlineStr"/>
-      <c r="J90" t="inlineStr"/>
-      <c r="K90" t="inlineStr"/>
-      <c r="L90" t="inlineStr"/>
       <c r="M90" t="n">
         <v>1</v>
       </c>
@@ -3625,10 +3269,6 @@
       <c r="H91" t="n">
         <v>1</v>
       </c>
-      <c r="I91" t="inlineStr"/>
-      <c r="J91" t="inlineStr"/>
-      <c r="K91" t="inlineStr"/>
-      <c r="L91" t="inlineStr"/>
       <c r="M91" t="n">
         <v>1</v>
       </c>
@@ -3660,10 +3300,6 @@
       <c r="H92" t="n">
         <v>2</v>
       </c>
-      <c r="I92" t="inlineStr"/>
-      <c r="J92" t="inlineStr"/>
-      <c r="K92" t="inlineStr"/>
-      <c r="L92" t="inlineStr"/>
       <c r="M92" t="n">
         <v>1</v>
       </c>
@@ -3695,10 +3331,6 @@
       <c r="H93" t="n">
         <v>3</v>
       </c>
-      <c r="I93" t="inlineStr"/>
-      <c r="J93" t="inlineStr"/>
-      <c r="K93" t="inlineStr"/>
-      <c r="L93" t="inlineStr"/>
       <c r="M93" t="n">
         <v>1</v>
       </c>
@@ -3730,10 +3362,6 @@
       <c r="H94" t="n">
         <v>1</v>
       </c>
-      <c r="I94" t="inlineStr"/>
-      <c r="J94" t="inlineStr"/>
-      <c r="K94" t="inlineStr"/>
-      <c r="L94" t="inlineStr"/>
       <c r="M94" t="n">
         <v>1</v>
       </c>
@@ -3765,10 +3393,6 @@
       <c r="H95" t="n">
         <v>2</v>
       </c>
-      <c r="I95" t="inlineStr"/>
-      <c r="J95" t="inlineStr"/>
-      <c r="K95" t="inlineStr"/>
-      <c r="L95" t="inlineStr"/>
       <c r="M95" t="n">
         <v>1</v>
       </c>
@@ -3800,10 +3424,6 @@
       <c r="H96" t="n">
         <v>1</v>
       </c>
-      <c r="I96" t="inlineStr"/>
-      <c r="J96" t="inlineStr"/>
-      <c r="K96" t="inlineStr"/>
-      <c r="L96" t="inlineStr"/>
       <c r="M96" t="n">
         <v>1</v>
       </c>
@@ -3835,10 +3455,6 @@
       <c r="H97" t="n">
         <v>2</v>
       </c>
-      <c r="I97" t="inlineStr"/>
-      <c r="J97" t="inlineStr"/>
-      <c r="K97" t="inlineStr"/>
-      <c r="L97" t="inlineStr"/>
       <c r="M97" t="n">
         <v>1</v>
       </c>
@@ -3870,10 +3486,6 @@
       <c r="H98" t="n">
         <v>3</v>
       </c>
-      <c r="I98" t="inlineStr"/>
-      <c r="J98" t="inlineStr"/>
-      <c r="K98" t="inlineStr"/>
-      <c r="L98" t="inlineStr"/>
       <c r="M98" t="n">
         <v>1</v>
       </c>
@@ -3905,10 +3517,6 @@
       <c r="H99" t="n">
         <v>1</v>
       </c>
-      <c r="I99" t="inlineStr"/>
-      <c r="J99" t="inlineStr"/>
-      <c r="K99" t="inlineStr"/>
-      <c r="L99" t="inlineStr"/>
       <c r="M99" t="n">
         <v>1</v>
       </c>
@@ -3940,10 +3548,6 @@
       <c r="H100" t="n">
         <v>2</v>
       </c>
-      <c r="I100" t="inlineStr"/>
-      <c r="J100" t="inlineStr"/>
-      <c r="K100" t="inlineStr"/>
-      <c r="L100" t="inlineStr"/>
       <c r="M100" t="n">
         <v>1</v>
       </c>
@@ -3975,10 +3579,6 @@
       <c r="H101" t="n">
         <v>1</v>
       </c>
-      <c r="I101" t="inlineStr"/>
-      <c r="J101" t="inlineStr"/>
-      <c r="K101" t="inlineStr"/>
-      <c r="L101" t="inlineStr"/>
       <c r="M101" t="n">
         <v>1</v>
       </c>
@@ -4010,10 +3610,6 @@
       <c r="H102" t="n">
         <v>2</v>
       </c>
-      <c r="I102" t="inlineStr"/>
-      <c r="J102" t="inlineStr"/>
-      <c r="K102" t="inlineStr"/>
-      <c r="L102" t="inlineStr"/>
       <c r="M102" t="n">
         <v>1</v>
       </c>
@@ -4045,10 +3641,6 @@
       <c r="H103" t="n">
         <v>2</v>
       </c>
-      <c r="I103" t="inlineStr"/>
-      <c r="J103" t="inlineStr"/>
-      <c r="K103" t="inlineStr"/>
-      <c r="L103" t="inlineStr"/>
       <c r="M103" t="n">
         <v>1</v>
       </c>
@@ -4080,10 +3672,6 @@
       <c r="H104" t="n">
         <v>3</v>
       </c>
-      <c r="I104" t="inlineStr"/>
-      <c r="J104" t="inlineStr"/>
-      <c r="K104" t="inlineStr"/>
-      <c r="L104" t="inlineStr"/>
       <c r="M104" t="n">
         <v>1</v>
       </c>
@@ -4115,10 +3703,6 @@
       <c r="H105" t="n">
         <v>1</v>
       </c>
-      <c r="I105" t="inlineStr"/>
-      <c r="J105" t="inlineStr"/>
-      <c r="K105" t="inlineStr"/>
-      <c r="L105" t="inlineStr"/>
       <c r="M105" t="n">
         <v>1</v>
       </c>
@@ -4150,10 +3734,6 @@
       <c r="H106" t="n">
         <v>2</v>
       </c>
-      <c r="I106" t="inlineStr"/>
-      <c r="J106" t="inlineStr"/>
-      <c r="K106" t="inlineStr"/>
-      <c r="L106" t="inlineStr"/>
       <c r="M106" t="n">
         <v>1</v>
       </c>
@@ -4185,10 +3765,6 @@
       <c r="H107" t="n">
         <v>2</v>
       </c>
-      <c r="I107" t="inlineStr"/>
-      <c r="J107" t="inlineStr"/>
-      <c r="K107" t="inlineStr"/>
-      <c r="L107" t="inlineStr"/>
       <c r="M107" t="n">
         <v>1</v>
       </c>
@@ -4220,10 +3796,6 @@
       <c r="H108" t="n">
         <v>2</v>
       </c>
-      <c r="I108" t="inlineStr"/>
-      <c r="J108" t="inlineStr"/>
-      <c r="K108" t="inlineStr"/>
-      <c r="L108" t="inlineStr"/>
       <c r="M108" t="n">
         <v>1</v>
       </c>
@@ -4255,10 +3827,6 @@
       <c r="H109" t="n">
         <v>2</v>
       </c>
-      <c r="I109" t="inlineStr"/>
-      <c r="J109" t="inlineStr"/>
-      <c r="K109" t="inlineStr"/>
-      <c r="L109" t="inlineStr"/>
       <c r="M109" t="n">
         <v>1</v>
       </c>
@@ -4290,10 +3858,6 @@
       <c r="H110" t="n">
         <v>2</v>
       </c>
-      <c r="I110" t="inlineStr"/>
-      <c r="J110" t="inlineStr"/>
-      <c r="K110" t="inlineStr"/>
-      <c r="L110" t="inlineStr"/>
       <c r="M110" t="n">
         <v>1</v>
       </c>
@@ -4325,10 +3889,6 @@
       <c r="H111" t="n">
         <v>2</v>
       </c>
-      <c r="I111" t="inlineStr"/>
-      <c r="J111" t="inlineStr"/>
-      <c r="K111" t="inlineStr"/>
-      <c r="L111" t="inlineStr"/>
       <c r="M111" t="n">
         <v>1</v>
       </c>
@@ -4360,10 +3920,6 @@
       <c r="H112" t="n">
         <v>2</v>
       </c>
-      <c r="I112" t="inlineStr"/>
-      <c r="J112" t="inlineStr"/>
-      <c r="K112" t="inlineStr"/>
-      <c r="L112" t="inlineStr"/>
       <c r="M112" t="n">
         <v>1</v>
       </c>
@@ -4395,10 +3951,6 @@
       <c r="H113" t="n">
         <v>2</v>
       </c>
-      <c r="I113" t="inlineStr"/>
-      <c r="J113" t="inlineStr"/>
-      <c r="K113" t="inlineStr"/>
-      <c r="L113" t="inlineStr"/>
       <c r="M113" t="n">
         <v>1</v>
       </c>
@@ -4430,10 +3982,6 @@
       <c r="H114" t="n">
         <v>1</v>
       </c>
-      <c r="I114" t="inlineStr"/>
-      <c r="J114" t="inlineStr"/>
-      <c r="K114" t="inlineStr"/>
-      <c r="L114" t="inlineStr"/>
       <c r="M114" t="n">
         <v>1</v>
       </c>
@@ -4465,10 +4013,6 @@
       <c r="H115" t="n">
         <v>2</v>
       </c>
-      <c r="I115" t="inlineStr"/>
-      <c r="J115" t="inlineStr"/>
-      <c r="K115" t="inlineStr"/>
-      <c r="L115" t="inlineStr"/>
       <c r="M115" t="n">
         <v>1</v>
       </c>
@@ -4500,10 +4044,6 @@
       <c r="H116" t="n">
         <v>2</v>
       </c>
-      <c r="I116" t="inlineStr"/>
-      <c r="J116" t="inlineStr"/>
-      <c r="K116" t="inlineStr"/>
-      <c r="L116" t="inlineStr"/>
       <c r="M116" t="n">
         <v>1</v>
       </c>
@@ -4535,10 +4075,6 @@
       <c r="H117" t="n">
         <v>2</v>
       </c>
-      <c r="I117" t="inlineStr"/>
-      <c r="J117" t="inlineStr"/>
-      <c r="K117" t="inlineStr"/>
-      <c r="L117" t="inlineStr"/>
       <c r="M117" t="n">
         <v>1</v>
       </c>
@@ -4570,10 +4106,6 @@
       <c r="H118" t="n">
         <v>2</v>
       </c>
-      <c r="I118" t="inlineStr"/>
-      <c r="J118" t="inlineStr"/>
-      <c r="K118" t="inlineStr"/>
-      <c r="L118" t="inlineStr"/>
       <c r="M118" t="n">
         <v>1</v>
       </c>
@@ -4605,10 +4137,6 @@
       <c r="H119" t="n">
         <v>2</v>
       </c>
-      <c r="I119" t="inlineStr"/>
-      <c r="J119" t="inlineStr"/>
-      <c r="K119" t="inlineStr"/>
-      <c r="L119" t="inlineStr"/>
       <c r="M119" t="n">
         <v>1</v>
       </c>
@@ -4640,10 +4168,6 @@
       <c r="H120" t="n">
         <v>2</v>
       </c>
-      <c r="I120" t="inlineStr"/>
-      <c r="J120" t="inlineStr"/>
-      <c r="K120" t="inlineStr"/>
-      <c r="L120" t="inlineStr"/>
       <c r="M120" t="n">
         <v>1</v>
       </c>
@@ -4675,10 +4199,6 @@
       <c r="H121" t="n">
         <v>2</v>
       </c>
-      <c r="I121" t="inlineStr"/>
-      <c r="J121" t="inlineStr"/>
-      <c r="K121" t="inlineStr"/>
-      <c r="L121" t="inlineStr"/>
       <c r="M121" t="n">
         <v>1</v>
       </c>
@@ -4710,10 +4230,6 @@
       <c r="H122" t="n">
         <v>2</v>
       </c>
-      <c r="I122" t="inlineStr"/>
-      <c r="J122" t="inlineStr"/>
-      <c r="K122" t="inlineStr"/>
-      <c r="L122" t="inlineStr"/>
       <c r="M122" t="n">
         <v>1</v>
       </c>
@@ -4745,10 +4261,6 @@
       <c r="H123" t="n">
         <v>3</v>
       </c>
-      <c r="I123" t="inlineStr"/>
-      <c r="J123" t="inlineStr"/>
-      <c r="K123" t="inlineStr"/>
-      <c r="L123" t="inlineStr"/>
       <c r="M123" t="n">
         <v>1</v>
       </c>
@@ -4780,10 +4292,6 @@
       <c r="H124" t="n">
         <v>3</v>
       </c>
-      <c r="I124" t="inlineStr"/>
-      <c r="J124" t="inlineStr"/>
-      <c r="K124" t="inlineStr"/>
-      <c r="L124" t="inlineStr"/>
       <c r="M124" t="n">
         <v>1</v>
       </c>
@@ -4815,10 +4323,6 @@
       <c r="H125" t="n">
         <v>1</v>
       </c>
-      <c r="I125" t="inlineStr"/>
-      <c r="J125" t="inlineStr"/>
-      <c r="K125" t="inlineStr"/>
-      <c r="L125" t="inlineStr"/>
       <c r="M125" t="n">
         <v>1</v>
       </c>
@@ -4850,10 +4354,6 @@
       <c r="H126" t="n">
         <v>3</v>
       </c>
-      <c r="I126" t="inlineStr"/>
-      <c r="J126" t="inlineStr"/>
-      <c r="K126" t="inlineStr"/>
-      <c r="L126" t="inlineStr"/>
       <c r="M126" t="n">
         <v>1</v>
       </c>
@@ -4885,10 +4385,6 @@
       <c r="H127" t="n">
         <v>3</v>
       </c>
-      <c r="I127" t="inlineStr"/>
-      <c r="J127" t="inlineStr"/>
-      <c r="K127" t="inlineStr"/>
-      <c r="L127" t="inlineStr"/>
       <c r="M127" t="n">
         <v>1</v>
       </c>
@@ -4920,10 +4416,6 @@
       <c r="H128" t="n">
         <v>1</v>
       </c>
-      <c r="I128" t="inlineStr"/>
-      <c r="J128" t="inlineStr"/>
-      <c r="K128" t="inlineStr"/>
-      <c r="L128" t="inlineStr"/>
       <c r="M128" t="n">
         <v>1</v>
       </c>
@@ -4955,10 +4447,6 @@
       <c r="H129" t="n">
         <v>2</v>
       </c>
-      <c r="I129" t="inlineStr"/>
-      <c r="J129" t="inlineStr"/>
-      <c r="K129" t="inlineStr"/>
-      <c r="L129" t="inlineStr"/>
       <c r="M129" t="n">
         <v>1</v>
       </c>
@@ -4990,10 +4478,6 @@
       <c r="H130" t="n">
         <v>2</v>
       </c>
-      <c r="I130" t="inlineStr"/>
-      <c r="J130" t="inlineStr"/>
-      <c r="K130" t="inlineStr"/>
-      <c r="L130" t="inlineStr"/>
       <c r="M130" t="n">
         <v>1</v>
       </c>
@@ -5025,10 +4509,6 @@
       <c r="H131" t="n">
         <v>2</v>
       </c>
-      <c r="I131" t="inlineStr"/>
-      <c r="J131" t="inlineStr"/>
-      <c r="K131" t="inlineStr"/>
-      <c r="L131" t="inlineStr"/>
       <c r="M131" t="n">
         <v>1</v>
       </c>
@@ -5060,10 +4540,6 @@
       <c r="H132" t="n">
         <v>2</v>
       </c>
-      <c r="I132" t="inlineStr"/>
-      <c r="J132" t="inlineStr"/>
-      <c r="K132" t="inlineStr"/>
-      <c r="L132" t="inlineStr"/>
       <c r="M132" t="n">
         <v>1</v>
       </c>
@@ -5095,10 +4571,6 @@
       <c r="H133" t="n">
         <v>2</v>
       </c>
-      <c r="I133" t="inlineStr"/>
-      <c r="J133" t="inlineStr"/>
-      <c r="K133" t="inlineStr"/>
-      <c r="L133" t="inlineStr"/>
       <c r="M133" t="n">
         <v>1</v>
       </c>
@@ -5130,10 +4602,6 @@
       <c r="H134" t="n">
         <v>2</v>
       </c>
-      <c r="I134" t="inlineStr"/>
-      <c r="J134" t="inlineStr"/>
-      <c r="K134" t="inlineStr"/>
-      <c r="L134" t="inlineStr"/>
       <c r="M134" t="n">
         <v>1</v>
       </c>
@@ -5165,10 +4633,6 @@
       <c r="H135" t="n">
         <v>2</v>
       </c>
-      <c r="I135" t="inlineStr"/>
-      <c r="J135" t="inlineStr"/>
-      <c r="K135" t="inlineStr"/>
-      <c r="L135" t="inlineStr"/>
       <c r="M135" t="n">
         <v>1</v>
       </c>
@@ -5200,10 +4664,6 @@
       <c r="H136" t="n">
         <v>2</v>
       </c>
-      <c r="I136" t="inlineStr"/>
-      <c r="J136" t="inlineStr"/>
-      <c r="K136" t="inlineStr"/>
-      <c r="L136" t="inlineStr"/>
       <c r="M136" t="n">
         <v>1</v>
       </c>
@@ -5235,10 +4695,6 @@
       <c r="H137" t="n">
         <v>2</v>
       </c>
-      <c r="I137" t="inlineStr"/>
-      <c r="J137" t="inlineStr"/>
-      <c r="K137" t="inlineStr"/>
-      <c r="L137" t="inlineStr"/>
       <c r="M137" t="n">
         <v>1</v>
       </c>
@@ -5252,7 +4708,7 @@
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>Prepaid items</t>
+          <t>Prepaid Items</t>
         </is>
       </c>
       <c r="D138" t="n">
@@ -5270,10 +4726,6 @@
       <c r="H138" t="n">
         <v>2</v>
       </c>
-      <c r="I138" t="inlineStr"/>
-      <c r="J138" t="inlineStr"/>
-      <c r="K138" t="inlineStr"/>
-      <c r="L138" t="inlineStr"/>
       <c r="M138" t="n">
         <v>1</v>
       </c>
@@ -5305,10 +4757,6 @@
       <c r="H139" t="n">
         <v>2</v>
       </c>
-      <c r="I139" t="inlineStr"/>
-      <c r="J139" t="inlineStr"/>
-      <c r="K139" t="inlineStr"/>
-      <c r="L139" t="inlineStr"/>
       <c r="M139" t="n">
         <v>1</v>
       </c>
@@ -5340,10 +4788,6 @@
       <c r="H140" t="n">
         <v>2</v>
       </c>
-      <c r="I140" t="inlineStr"/>
-      <c r="J140" t="inlineStr"/>
-      <c r="K140" t="inlineStr"/>
-      <c r="L140" t="inlineStr"/>
       <c r="M140" t="n">
         <v>1</v>
       </c>
@@ -5375,10 +4819,6 @@
       <c r="H141" t="n">
         <v>2</v>
       </c>
-      <c r="I141" t="inlineStr"/>
-      <c r="J141" t="inlineStr"/>
-      <c r="K141" t="inlineStr"/>
-      <c r="L141" t="inlineStr"/>
       <c r="M141" t="n">
         <v>1</v>
       </c>
@@ -5410,10 +4850,6 @@
       <c r="H142" t="n">
         <v>2</v>
       </c>
-      <c r="I142" t="inlineStr"/>
-      <c r="J142" t="inlineStr"/>
-      <c r="K142" t="inlineStr"/>
-      <c r="L142" t="inlineStr"/>
       <c r="M142" t="n">
         <v>1</v>
       </c>
@@ -5445,10 +4881,6 @@
       <c r="H143" t="n">
         <v>2</v>
       </c>
-      <c r="I143" t="inlineStr"/>
-      <c r="J143" t="inlineStr"/>
-      <c r="K143" t="inlineStr"/>
-      <c r="L143" t="inlineStr"/>
       <c r="M143" t="n">
         <v>1</v>
       </c>
@@ -5480,10 +4912,6 @@
       <c r="H144" t="n">
         <v>2</v>
       </c>
-      <c r="I144" t="inlineStr"/>
-      <c r="J144" t="inlineStr"/>
-      <c r="K144" t="inlineStr"/>
-      <c r="L144" t="inlineStr"/>
       <c r="M144" t="n">
         <v>1</v>
       </c>
@@ -5515,10 +4943,6 @@
       <c r="H145" t="n">
         <v>2</v>
       </c>
-      <c r="I145" t="inlineStr"/>
-      <c r="J145" t="inlineStr"/>
-      <c r="K145" t="inlineStr"/>
-      <c r="L145" t="inlineStr"/>
       <c r="M145" t="n">
         <v>1</v>
       </c>
@@ -5550,10 +4974,6 @@
       <c r="H146" t="n">
         <v>3</v>
       </c>
-      <c r="I146" t="inlineStr"/>
-      <c r="J146" t="inlineStr"/>
-      <c r="K146" t="inlineStr"/>
-      <c r="L146" t="inlineStr"/>
       <c r="M146" t="n">
         <v>1</v>
       </c>
@@ -5585,10 +5005,6 @@
       <c r="H147" t="n">
         <v>3</v>
       </c>
-      <c r="I147" t="inlineStr"/>
-      <c r="J147" t="inlineStr"/>
-      <c r="K147" t="inlineStr"/>
-      <c r="L147" t="inlineStr"/>
       <c r="M147" t="n">
         <v>1</v>
       </c>
@@ -5620,10 +5036,6 @@
       <c r="H148" t="n">
         <v>3</v>
       </c>
-      <c r="I148" t="inlineStr"/>
-      <c r="J148" t="inlineStr"/>
-      <c r="K148" t="inlineStr"/>
-      <c r="L148" t="inlineStr"/>
       <c r="M148" t="n">
         <v>1</v>
       </c>
@@ -5655,10 +5067,6 @@
       <c r="H149" t="n">
         <v>3</v>
       </c>
-      <c r="I149" t="inlineStr"/>
-      <c r="J149" t="inlineStr"/>
-      <c r="K149" t="inlineStr"/>
-      <c r="L149" t="inlineStr"/>
       <c r="M149" t="n">
         <v>1</v>
       </c>
@@ -5690,10 +5098,6 @@
       <c r="H150" t="n">
         <v>3</v>
       </c>
-      <c r="I150" t="inlineStr"/>
-      <c r="J150" t="inlineStr"/>
-      <c r="K150" t="inlineStr"/>
-      <c r="L150" t="inlineStr"/>
       <c r="M150" t="n">
         <v>1</v>
       </c>
@@ -5725,10 +5129,6 @@
       <c r="H151" t="n">
         <v>3</v>
       </c>
-      <c r="I151" t="inlineStr"/>
-      <c r="J151" t="inlineStr"/>
-      <c r="K151" t="inlineStr"/>
-      <c r="L151" t="inlineStr"/>
       <c r="M151" t="n">
         <v>1</v>
       </c>
@@ -5760,10 +5160,6 @@
       <c r="H152" t="n">
         <v>3</v>
       </c>
-      <c r="I152" t="inlineStr"/>
-      <c r="J152" t="inlineStr"/>
-      <c r="K152" t="inlineStr"/>
-      <c r="L152" t="inlineStr"/>
       <c r="M152" t="n">
         <v>1</v>
       </c>
@@ -5795,10 +5191,6 @@
       <c r="H153" t="n">
         <v>3</v>
       </c>
-      <c r="I153" t="inlineStr"/>
-      <c r="J153" t="inlineStr"/>
-      <c r="K153" t="inlineStr"/>
-      <c r="L153" t="inlineStr"/>
       <c r="M153" t="n">
         <v>1</v>
       </c>
@@ -5830,10 +5222,6 @@
       <c r="H154" t="n">
         <v>1</v>
       </c>
-      <c r="I154" t="inlineStr"/>
-      <c r="J154" t="inlineStr"/>
-      <c r="K154" t="inlineStr"/>
-      <c r="L154" t="inlineStr"/>
       <c r="M154" t="n">
         <v>1</v>
       </c>
@@ -5865,10 +5253,6 @@
       <c r="H155" t="n">
         <v>2</v>
       </c>
-      <c r="I155" t="inlineStr"/>
-      <c r="J155" t="inlineStr"/>
-      <c r="K155" t="inlineStr"/>
-      <c r="L155" t="inlineStr"/>
       <c r="M155" t="n">
         <v>1</v>
       </c>
@@ -5900,10 +5284,6 @@
       <c r="H156" t="n">
         <v>3</v>
       </c>
-      <c r="I156" t="inlineStr"/>
-      <c r="J156" t="inlineStr"/>
-      <c r="K156" t="inlineStr"/>
-      <c r="L156" t="inlineStr"/>
       <c r="M156" t="n">
         <v>1</v>
       </c>
@@ -5935,10 +5315,6 @@
       <c r="H157" t="n">
         <v>3</v>
       </c>
-      <c r="I157" t="inlineStr"/>
-      <c r="J157" t="inlineStr"/>
-      <c r="K157" t="inlineStr"/>
-      <c r="L157" t="inlineStr"/>
       <c r="M157" t="n">
         <v>1</v>
       </c>
@@ -5970,10 +5346,6 @@
       <c r="H158" t="n">
         <v>1</v>
       </c>
-      <c r="I158" t="inlineStr"/>
-      <c r="J158" t="inlineStr"/>
-      <c r="K158" t="inlineStr"/>
-      <c r="L158" t="inlineStr"/>
       <c r="M158" t="n">
         <v>1</v>
       </c>
@@ -6005,10 +5377,6 @@
       <c r="H159" t="n">
         <v>2</v>
       </c>
-      <c r="I159" t="inlineStr"/>
-      <c r="J159" t="inlineStr"/>
-      <c r="K159" t="inlineStr"/>
-      <c r="L159" t="inlineStr"/>
       <c r="M159" t="n">
         <v>1</v>
       </c>
@@ -6040,10 +5408,6 @@
       <c r="H160" t="n">
         <v>2</v>
       </c>
-      <c r="I160" t="inlineStr"/>
-      <c r="J160" t="inlineStr"/>
-      <c r="K160" t="inlineStr"/>
-      <c r="L160" t="inlineStr"/>
       <c r="M160" t="n">
         <v>1</v>
       </c>
@@ -6075,10 +5439,6 @@
       <c r="H161" t="n">
         <v>2</v>
       </c>
-      <c r="I161" t="inlineStr"/>
-      <c r="J161" t="inlineStr"/>
-      <c r="K161" t="inlineStr"/>
-      <c r="L161" t="inlineStr"/>
       <c r="M161" t="n">
         <v>1</v>
       </c>
@@ -6110,10 +5470,6 @@
       <c r="H162" t="n">
         <v>2</v>
       </c>
-      <c r="I162" t="inlineStr"/>
-      <c r="J162" t="inlineStr"/>
-      <c r="K162" t="inlineStr"/>
-      <c r="L162" t="inlineStr"/>
       <c r="M162" t="n">
         <v>1</v>
       </c>
@@ -6145,10 +5501,6 @@
       <c r="H163" t="n">
         <v>2</v>
       </c>
-      <c r="I163" t="inlineStr"/>
-      <c r="J163" t="inlineStr"/>
-      <c r="K163" t="inlineStr"/>
-      <c r="L163" t="inlineStr"/>
       <c r="M163" t="n">
         <v>1</v>
       </c>
@@ -6180,10 +5532,6 @@
       <c r="H164" t="n">
         <v>2</v>
       </c>
-      <c r="I164" t="inlineStr"/>
-      <c r="J164" t="inlineStr"/>
-      <c r="K164" t="inlineStr"/>
-      <c r="L164" t="inlineStr"/>
       <c r="M164" t="n">
         <v>1</v>
       </c>
@@ -6215,10 +5563,6 @@
       <c r="H165" t="n">
         <v>2</v>
       </c>
-      <c r="I165" t="inlineStr"/>
-      <c r="J165" t="inlineStr"/>
-      <c r="K165" t="inlineStr"/>
-      <c r="L165" t="inlineStr"/>
       <c r="M165" t="n">
         <v>1</v>
       </c>
@@ -6250,10 +5594,6 @@
       <c r="H166" t="n">
         <v>2</v>
       </c>
-      <c r="I166" t="inlineStr"/>
-      <c r="J166" t="inlineStr"/>
-      <c r="K166" t="inlineStr"/>
-      <c r="L166" t="inlineStr"/>
       <c r="M166" t="n">
         <v>1</v>
       </c>
@@ -6285,10 +5625,6 @@
       <c r="H167" t="n">
         <v>2</v>
       </c>
-      <c r="I167" t="inlineStr"/>
-      <c r="J167" t="inlineStr"/>
-      <c r="K167" t="inlineStr"/>
-      <c r="L167" t="inlineStr"/>
       <c r="M167" t="n">
         <v>1</v>
       </c>
@@ -6320,10 +5656,6 @@
       <c r="H168" t="n">
         <v>2</v>
       </c>
-      <c r="I168" t="inlineStr"/>
-      <c r="J168" t="inlineStr"/>
-      <c r="K168" t="inlineStr"/>
-      <c r="L168" t="inlineStr"/>
       <c r="M168" t="n">
         <v>1</v>
       </c>
@@ -6355,10 +5687,6 @@
       <c r="H169" t="n">
         <v>2</v>
       </c>
-      <c r="I169" t="inlineStr"/>
-      <c r="J169" t="inlineStr"/>
-      <c r="K169" t="inlineStr"/>
-      <c r="L169" t="inlineStr"/>
       <c r="M169" t="n">
         <v>1</v>
       </c>
@@ -6390,10 +5718,6 @@
       <c r="H170" t="n">
         <v>2</v>
       </c>
-      <c r="I170" t="inlineStr"/>
-      <c r="J170" t="inlineStr"/>
-      <c r="K170" t="inlineStr"/>
-      <c r="L170" t="inlineStr"/>
       <c r="M170" t="n">
         <v>1</v>
       </c>
@@ -6425,10 +5749,6 @@
       <c r="H171" t="n">
         <v>2</v>
       </c>
-      <c r="I171" t="inlineStr"/>
-      <c r="J171" t="inlineStr"/>
-      <c r="K171" t="inlineStr"/>
-      <c r="L171" t="inlineStr"/>
       <c r="M171" t="n">
         <v>1</v>
       </c>
@@ -6460,10 +5780,6 @@
       <c r="H172" t="n">
         <v>2</v>
       </c>
-      <c r="I172" t="inlineStr"/>
-      <c r="J172" t="inlineStr"/>
-      <c r="K172" t="inlineStr"/>
-      <c r="L172" t="inlineStr"/>
       <c r="M172" t="n">
         <v>1</v>
       </c>
@@ -6495,10 +5811,6 @@
       <c r="H173" t="n">
         <v>2</v>
       </c>
-      <c r="I173" t="inlineStr"/>
-      <c r="J173" t="inlineStr"/>
-      <c r="K173" t="inlineStr"/>
-      <c r="L173" t="inlineStr"/>
       <c r="M173" t="n">
         <v>1</v>
       </c>
@@ -6530,10 +5842,6 @@
       <c r="H174" t="n">
         <v>2</v>
       </c>
-      <c r="I174" t="inlineStr"/>
-      <c r="J174" t="inlineStr"/>
-      <c r="K174" t="inlineStr"/>
-      <c r="L174" t="inlineStr"/>
       <c r="M174" t="n">
         <v>1</v>
       </c>
@@ -6565,10 +5873,6 @@
       <c r="H175" t="n">
         <v>2</v>
       </c>
-      <c r="I175" t="inlineStr"/>
-      <c r="J175" t="inlineStr"/>
-      <c r="K175" t="inlineStr"/>
-      <c r="L175" t="inlineStr"/>
       <c r="M175" t="n">
         <v>1</v>
       </c>
@@ -6600,10 +5904,6 @@
       <c r="H176" t="n">
         <v>3</v>
       </c>
-      <c r="I176" t="inlineStr"/>
-      <c r="J176" t="inlineStr"/>
-      <c r="K176" t="inlineStr"/>
-      <c r="L176" t="inlineStr"/>
       <c r="M176" t="n">
         <v>1</v>
       </c>
@@ -6635,10 +5935,6 @@
       <c r="H177" t="n">
         <v>3</v>
       </c>
-      <c r="I177" t="inlineStr"/>
-      <c r="J177" t="inlineStr"/>
-      <c r="K177" t="inlineStr"/>
-      <c r="L177" t="inlineStr"/>
       <c r="M177" t="n">
         <v>1</v>
       </c>
@@ -6670,10 +5966,6 @@
       <c r="H178" t="n">
         <v>3</v>
       </c>
-      <c r="I178" t="inlineStr"/>
-      <c r="J178" t="inlineStr"/>
-      <c r="K178" t="inlineStr"/>
-      <c r="L178" t="inlineStr"/>
       <c r="M178" t="n">
         <v>1</v>
       </c>
@@ -6705,10 +5997,6 @@
       <c r="H179" t="n">
         <v>1</v>
       </c>
-      <c r="I179" t="inlineStr"/>
-      <c r="J179" t="inlineStr"/>
-      <c r="K179" t="inlineStr"/>
-      <c r="L179" t="inlineStr"/>
       <c r="M179" t="n">
         <v>1</v>
       </c>
@@ -6740,10 +6028,6 @@
       <c r="H180" t="n">
         <v>2</v>
       </c>
-      <c r="I180" t="inlineStr"/>
-      <c r="J180" t="inlineStr"/>
-      <c r="K180" t="inlineStr"/>
-      <c r="L180" t="inlineStr"/>
       <c r="M180" t="n">
         <v>1</v>
       </c>
@@ -6775,10 +6059,6 @@
       <c r="H181" t="n">
         <v>3</v>
       </c>
-      <c r="I181" t="inlineStr"/>
-      <c r="J181" t="inlineStr"/>
-      <c r="K181" t="inlineStr"/>
-      <c r="L181" t="inlineStr"/>
       <c r="M181" t="n">
         <v>1</v>
       </c>
@@ -6810,10 +6090,6 @@
       <c r="H182" t="n">
         <v>3</v>
       </c>
-      <c r="I182" t="inlineStr"/>
-      <c r="J182" t="inlineStr"/>
-      <c r="K182" t="inlineStr"/>
-      <c r="L182" t="inlineStr"/>
       <c r="M182" t="n">
         <v>1</v>
       </c>
@@ -6845,10 +6121,6 @@
       <c r="H183" t="n">
         <v>1</v>
       </c>
-      <c r="I183" t="inlineStr"/>
-      <c r="J183" t="inlineStr"/>
-      <c r="K183" t="inlineStr"/>
-      <c r="L183" t="inlineStr"/>
       <c r="M183" t="n">
         <v>1</v>
       </c>
@@ -6880,10 +6152,6 @@
       <c r="H184" t="n">
         <v>2</v>
       </c>
-      <c r="I184" t="inlineStr"/>
-      <c r="J184" t="inlineStr"/>
-      <c r="K184" t="inlineStr"/>
-      <c r="L184" t="inlineStr"/>
       <c r="M184" t="n">
         <v>1</v>
       </c>
@@ -6915,10 +6183,6 @@
       <c r="H185" t="n">
         <v>2</v>
       </c>
-      <c r="I185" t="inlineStr"/>
-      <c r="J185" t="inlineStr"/>
-      <c r="K185" t="inlineStr"/>
-      <c r="L185" t="inlineStr"/>
       <c r="M185" t="n">
         <v>1</v>
       </c>
@@ -6950,10 +6214,6 @@
       <c r="H186" t="n">
         <v>2</v>
       </c>
-      <c r="I186" t="inlineStr"/>
-      <c r="J186" t="inlineStr"/>
-      <c r="K186" t="inlineStr"/>
-      <c r="L186" t="inlineStr"/>
       <c r="M186" t="n">
         <v>1</v>
       </c>
@@ -6985,10 +6245,6 @@
       <c r="H187" t="n">
         <v>3</v>
       </c>
-      <c r="I187" t="inlineStr"/>
-      <c r="J187" t="inlineStr"/>
-      <c r="K187" t="inlineStr"/>
-      <c r="L187" t="inlineStr"/>
       <c r="M187" t="n">
         <v>1</v>
       </c>
@@ -7020,10 +6276,6 @@
       <c r="H188" t="n">
         <v>3</v>
       </c>
-      <c r="I188" t="inlineStr"/>
-      <c r="J188" t="inlineStr"/>
-      <c r="K188" t="inlineStr"/>
-      <c r="L188" t="inlineStr"/>
       <c r="M188" t="n">
         <v>1</v>
       </c>
@@ -7055,10 +6307,6 @@
       <c r="H189" t="n">
         <v>3</v>
       </c>
-      <c r="I189" t="inlineStr"/>
-      <c r="J189" t="inlineStr"/>
-      <c r="K189" t="inlineStr"/>
-      <c r="L189" t="inlineStr"/>
       <c r="M189" t="n">
         <v>1</v>
       </c>
@@ -7090,10 +6338,6 @@
       <c r="H190" t="n">
         <v>3</v>
       </c>
-      <c r="I190" t="inlineStr"/>
-      <c r="J190" t="inlineStr"/>
-      <c r="K190" t="inlineStr"/>
-      <c r="L190" t="inlineStr"/>
       <c r="M190" t="n">
         <v>1</v>
       </c>
@@ -7107,7 +6351,7 @@
       </c>
       <c r="C191" t="inlineStr">
         <is>
-          <t>Total Liabilities, Deferred inflows of resources, and Net position</t>
+          <t>Total Liabilities, Deferred Inflows of Resources, and Net Position</t>
         </is>
       </c>
       <c r="D191" t="n">
@@ -7125,10 +6369,6 @@
       <c r="H191" t="n">
         <v>3</v>
       </c>
-      <c r="I191" t="inlineStr"/>
-      <c r="J191" t="inlineStr"/>
-      <c r="K191" t="inlineStr"/>
-      <c r="L191" t="inlineStr"/>
       <c r="M191" t="n">
         <v>1</v>
       </c>
@@ -7160,10 +6400,6 @@
       <c r="H192" t="n">
         <v>1</v>
       </c>
-      <c r="I192" t="inlineStr"/>
-      <c r="J192" t="inlineStr"/>
-      <c r="K192" t="inlineStr"/>
-      <c r="L192" t="inlineStr"/>
       <c r="M192" t="n">
         <v>1</v>
       </c>
@@ -7195,10 +6431,6 @@
       <c r="H193" t="n">
         <v>2</v>
       </c>
-      <c r="I193" t="inlineStr"/>
-      <c r="J193" t="inlineStr"/>
-      <c r="K193" t="inlineStr"/>
-      <c r="L193" t="inlineStr"/>
       <c r="M193" t="n">
         <v>1</v>
       </c>
@@ -7230,10 +6462,6 @@
       <c r="H194" t="n">
         <v>2</v>
       </c>
-      <c r="I194" t="inlineStr"/>
-      <c r="J194" t="inlineStr"/>
-      <c r="K194" t="inlineStr"/>
-      <c r="L194" t="inlineStr"/>
       <c r="M194" t="n">
         <v>1</v>
       </c>
@@ -7265,10 +6493,6 @@
       <c r="H195" t="n">
         <v>2</v>
       </c>
-      <c r="I195" t="inlineStr"/>
-      <c r="J195" t="inlineStr"/>
-      <c r="K195" t="inlineStr"/>
-      <c r="L195" t="inlineStr"/>
       <c r="M195" t="n">
         <v>1</v>
       </c>
@@ -7300,10 +6524,6 @@
       <c r="H196" t="n">
         <v>2</v>
       </c>
-      <c r="I196" t="inlineStr"/>
-      <c r="J196" t="inlineStr"/>
-      <c r="K196" t="inlineStr"/>
-      <c r="L196" t="inlineStr"/>
       <c r="M196" t="n">
         <v>1</v>
       </c>
@@ -7335,10 +6555,6 @@
       <c r="H197" t="n">
         <v>2</v>
       </c>
-      <c r="I197" t="inlineStr"/>
-      <c r="J197" t="inlineStr"/>
-      <c r="K197" t="inlineStr"/>
-      <c r="L197" t="inlineStr"/>
       <c r="M197" t="n">
         <v>1</v>
       </c>
@@ -7370,10 +6586,6 @@
       <c r="H198" t="n">
         <v>3</v>
       </c>
-      <c r="I198" t="inlineStr"/>
-      <c r="J198" t="inlineStr"/>
-      <c r="K198" t="inlineStr"/>
-      <c r="L198" t="inlineStr"/>
       <c r="M198" t="n">
         <v>1</v>
       </c>
@@ -7405,10 +6617,6 @@
       <c r="H199" t="n">
         <v>3</v>
       </c>
-      <c r="I199" t="inlineStr"/>
-      <c r="J199" t="inlineStr"/>
-      <c r="K199" t="inlineStr"/>
-      <c r="L199" t="inlineStr"/>
       <c r="M199" t="n">
         <v>1</v>
       </c>
@@ -7440,10 +6648,6 @@
       <c r="H200" t="n">
         <v>3</v>
       </c>
-      <c r="I200" t="inlineStr"/>
-      <c r="J200" t="inlineStr"/>
-      <c r="K200" t="inlineStr"/>
-      <c r="L200" t="inlineStr"/>
       <c r="M200" t="n">
         <v>1</v>
       </c>
@@ -7475,10 +6679,6 @@
       <c r="H201" t="n">
         <v>1</v>
       </c>
-      <c r="I201" t="inlineStr"/>
-      <c r="J201" t="inlineStr"/>
-      <c r="K201" t="inlineStr"/>
-      <c r="L201" t="inlineStr"/>
       <c r="M201" t="n">
         <v>1</v>
       </c>
@@ -7510,10 +6710,6 @@
       <c r="H202" t="n">
         <v>2</v>
       </c>
-      <c r="I202" t="inlineStr"/>
-      <c r="J202" t="inlineStr"/>
-      <c r="K202" t="inlineStr"/>
-      <c r="L202" t="inlineStr"/>
       <c r="M202" t="n">
         <v>1</v>
       </c>
@@ -7545,10 +6741,6 @@
       <c r="H203" t="n">
         <v>2</v>
       </c>
-      <c r="I203" t="inlineStr"/>
-      <c r="J203" t="inlineStr"/>
-      <c r="K203" t="inlineStr"/>
-      <c r="L203" t="inlineStr"/>
       <c r="M203" t="n">
         <v>1</v>
       </c>
@@ -7580,10 +6772,6 @@
       <c r="H204" t="n">
         <v>2</v>
       </c>
-      <c r="I204" t="inlineStr"/>
-      <c r="J204" t="inlineStr"/>
-      <c r="K204" t="inlineStr"/>
-      <c r="L204" t="inlineStr"/>
       <c r="M204" t="n">
         <v>1</v>
       </c>
@@ -7615,10 +6803,6 @@
       <c r="H205" t="n">
         <v>2</v>
       </c>
-      <c r="I205" t="inlineStr"/>
-      <c r="J205" t="inlineStr"/>
-      <c r="K205" t="inlineStr"/>
-      <c r="L205" t="inlineStr"/>
       <c r="M205" t="n">
         <v>1</v>
       </c>
@@ -7650,10 +6834,6 @@
       <c r="H206" t="n">
         <v>2</v>
       </c>
-      <c r="I206" t="inlineStr"/>
-      <c r="J206" t="inlineStr"/>
-      <c r="K206" t="inlineStr"/>
-      <c r="L206" t="inlineStr"/>
       <c r="M206" t="n">
         <v>1</v>
       </c>
@@ -7685,10 +6865,6 @@
       <c r="H207" t="n">
         <v>2</v>
       </c>
-      <c r="I207" t="inlineStr"/>
-      <c r="J207" t="inlineStr"/>
-      <c r="K207" t="inlineStr"/>
-      <c r="L207" t="inlineStr"/>
       <c r="M207" t="n">
         <v>1</v>
       </c>
@@ -7720,10 +6896,6 @@
       <c r="H208" t="n">
         <v>2</v>
       </c>
-      <c r="I208" t="inlineStr"/>
-      <c r="J208" t="inlineStr"/>
-      <c r="K208" t="inlineStr"/>
-      <c r="L208" t="inlineStr"/>
       <c r="M208" t="n">
         <v>1</v>
       </c>
@@ -7755,10 +6927,6 @@
       <c r="H209" t="n">
         <v>2</v>
       </c>
-      <c r="I209" t="inlineStr"/>
-      <c r="J209" t="inlineStr"/>
-      <c r="K209" t="inlineStr"/>
-      <c r="L209" t="inlineStr"/>
       <c r="M209" t="n">
         <v>1</v>
       </c>
@@ -7790,10 +6958,6 @@
       <c r="H210" t="n">
         <v>2</v>
       </c>
-      <c r="I210" t="inlineStr"/>
-      <c r="J210" t="inlineStr"/>
-      <c r="K210" t="inlineStr"/>
-      <c r="L210" t="inlineStr"/>
       <c r="M210" t="n">
         <v>1</v>
       </c>
@@ -7825,10 +6989,6 @@
       <c r="H211" t="n">
         <v>3</v>
       </c>
-      <c r="I211" t="inlineStr"/>
-      <c r="J211" t="inlineStr"/>
-      <c r="K211" t="inlineStr"/>
-      <c r="L211" t="inlineStr"/>
       <c r="M211" t="n">
         <v>1</v>
       </c>
@@ -7860,10 +7020,6 @@
       <c r="H212" t="n">
         <v>1</v>
       </c>
-      <c r="I212" t="inlineStr"/>
-      <c r="J212" t="inlineStr"/>
-      <c r="K212" t="inlineStr"/>
-      <c r="L212" t="inlineStr"/>
       <c r="M212" t="n">
         <v>1</v>
       </c>
@@ -7895,10 +7051,6 @@
       <c r="H213" t="n">
         <v>2</v>
       </c>
-      <c r="I213" t="inlineStr"/>
-      <c r="J213" t="inlineStr"/>
-      <c r="K213" t="inlineStr"/>
-      <c r="L213" t="inlineStr"/>
       <c r="M213" t="n">
         <v>1</v>
       </c>
@@ -7930,10 +7082,6 @@
       <c r="H214" t="n">
         <v>2</v>
       </c>
-      <c r="I214" t="inlineStr"/>
-      <c r="J214" t="inlineStr"/>
-      <c r="K214" t="inlineStr"/>
-      <c r="L214" t="inlineStr"/>
       <c r="M214" t="n">
         <v>1</v>
       </c>
@@ -7965,10 +7113,6 @@
       <c r="H215" t="n">
         <v>2</v>
       </c>
-      <c r="I215" t="inlineStr"/>
-      <c r="J215" t="inlineStr"/>
-      <c r="K215" t="inlineStr"/>
-      <c r="L215" t="inlineStr"/>
       <c r="M215" t="n">
         <v>1</v>
       </c>
@@ -8000,10 +7144,6 @@
       <c r="H216" t="n">
         <v>2</v>
       </c>
-      <c r="I216" t="inlineStr"/>
-      <c r="J216" t="inlineStr"/>
-      <c r="K216" t="inlineStr"/>
-      <c r="L216" t="inlineStr"/>
       <c r="M216" t="n">
         <v>1</v>
       </c>
@@ -8035,10 +7175,6 @@
       <c r="H217" t="n">
         <v>2</v>
       </c>
-      <c r="I217" t="inlineStr"/>
-      <c r="J217" t="inlineStr"/>
-      <c r="K217" t="inlineStr"/>
-      <c r="L217" t="inlineStr"/>
       <c r="M217" t="n">
         <v>1</v>
       </c>
@@ -8070,10 +7206,6 @@
       <c r="H218" t="n">
         <v>2</v>
       </c>
-      <c r="I218" t="inlineStr"/>
-      <c r="J218" t="inlineStr"/>
-      <c r="K218" t="inlineStr"/>
-      <c r="L218" t="inlineStr"/>
       <c r="M218" t="n">
         <v>1</v>
       </c>
@@ -8105,10 +7237,6 @@
       <c r="H219" t="n">
         <v>2</v>
       </c>
-      <c r="I219" t="inlineStr"/>
-      <c r="J219" t="inlineStr"/>
-      <c r="K219" t="inlineStr"/>
-      <c r="L219" t="inlineStr"/>
       <c r="M219" t="n">
         <v>1</v>
       </c>
@@ -8140,10 +7268,6 @@
       <c r="H220" t="n">
         <v>2</v>
       </c>
-      <c r="I220" t="inlineStr"/>
-      <c r="J220" t="inlineStr"/>
-      <c r="K220" t="inlineStr"/>
-      <c r="L220" t="inlineStr"/>
       <c r="M220" t="n">
         <v>1</v>
       </c>
@@ -8175,10 +7299,6 @@
       <c r="H221" t="n">
         <v>2</v>
       </c>
-      <c r="I221" t="inlineStr"/>
-      <c r="J221" t="inlineStr"/>
-      <c r="K221" t="inlineStr"/>
-      <c r="L221" t="inlineStr"/>
       <c r="M221" t="n">
         <v>1</v>
       </c>
@@ -8210,10 +7330,6 @@
       <c r="H222" t="n">
         <v>2</v>
       </c>
-      <c r="I222" t="inlineStr"/>
-      <c r="J222" t="inlineStr"/>
-      <c r="K222" t="inlineStr"/>
-      <c r="L222" t="inlineStr"/>
       <c r="M222" t="n">
         <v>1</v>
       </c>
@@ -8245,10 +7361,6 @@
       <c r="H223" t="n">
         <v>3</v>
       </c>
-      <c r="I223" t="inlineStr"/>
-      <c r="J223" t="inlineStr"/>
-      <c r="K223" t="inlineStr"/>
-      <c r="L223" t="inlineStr"/>
       <c r="M223" t="n">
         <v>1</v>
       </c>
@@ -8280,10 +7392,6 @@
       <c r="H224" t="n">
         <v>3</v>
       </c>
-      <c r="I224" t="inlineStr"/>
-      <c r="J224" t="inlineStr"/>
-      <c r="K224" t="inlineStr"/>
-      <c r="L224" t="inlineStr"/>
       <c r="M224" t="n">
         <v>1</v>
       </c>
@@ -8315,10 +7423,6 @@
       <c r="H225" t="n">
         <v>1</v>
       </c>
-      <c r="I225" t="inlineStr"/>
-      <c r="J225" t="inlineStr"/>
-      <c r="K225" t="inlineStr"/>
-      <c r="L225" t="inlineStr"/>
       <c r="M225" t="n">
         <v>1</v>
       </c>
@@ -8350,10 +7454,6 @@
       <c r="H226" t="n">
         <v>2</v>
       </c>
-      <c r="I226" t="inlineStr"/>
-      <c r="J226" t="inlineStr"/>
-      <c r="K226" t="inlineStr"/>
-      <c r="L226" t="inlineStr"/>
       <c r="M226" t="n">
         <v>1</v>
       </c>
@@ -8385,10 +7485,6 @@
       <c r="H227" t="n">
         <v>2</v>
       </c>
-      <c r="I227" t="inlineStr"/>
-      <c r="J227" t="inlineStr"/>
-      <c r="K227" t="inlineStr"/>
-      <c r="L227" t="inlineStr"/>
       <c r="M227" t="n">
         <v>1</v>
       </c>
@@ -8420,10 +7516,6 @@
       <c r="H228" t="n">
         <v>2</v>
       </c>
-      <c r="I228" t="inlineStr"/>
-      <c r="J228" t="inlineStr"/>
-      <c r="K228" t="inlineStr"/>
-      <c r="L228" t="inlineStr"/>
       <c r="M228" t="n">
         <v>1</v>
       </c>
@@ -8455,10 +7547,6 @@
       <c r="H229" t="n">
         <v>3</v>
       </c>
-      <c r="I229" t="inlineStr"/>
-      <c r="J229" t="inlineStr"/>
-      <c r="K229" t="inlineStr"/>
-      <c r="L229" t="inlineStr"/>
       <c r="M229" t="n">
         <v>1</v>
       </c>
@@ -8490,10 +7578,6 @@
       <c r="H230" t="n">
         <v>3</v>
       </c>
-      <c r="I230" t="inlineStr"/>
-      <c r="J230" t="inlineStr"/>
-      <c r="K230" t="inlineStr"/>
-      <c r="L230" t="inlineStr"/>
       <c r="M230" t="n">
         <v>1</v>
       </c>
@@ -8525,10 +7609,6 @@
       <c r="H231" t="n">
         <v>1</v>
       </c>
-      <c r="I231" t="inlineStr"/>
-      <c r="J231" t="inlineStr"/>
-      <c r="K231" t="inlineStr"/>
-      <c r="L231" t="inlineStr"/>
       <c r="M231" t="n">
         <v>1</v>
       </c>
@@ -8560,10 +7640,6 @@
       <c r="H232" t="n">
         <v>3</v>
       </c>
-      <c r="I232" t="inlineStr"/>
-      <c r="J232" t="inlineStr"/>
-      <c r="K232" t="inlineStr"/>
-      <c r="L232" t="inlineStr"/>
       <c r="M232" t="n">
         <v>1</v>
       </c>
@@ -8595,10 +7671,6 @@
       <c r="H233" t="n">
         <v>3</v>
       </c>
-      <c r="I233" t="inlineStr"/>
-      <c r="J233" t="inlineStr"/>
-      <c r="K233" t="inlineStr"/>
-      <c r="L233" t="inlineStr"/>
       <c r="M233" t="n">
         <v>1</v>
       </c>
@@ -8630,10 +7702,6 @@
       <c r="H234" t="n">
         <v>1</v>
       </c>
-      <c r="I234" t="inlineStr"/>
-      <c r="J234" t="inlineStr"/>
-      <c r="K234" t="inlineStr"/>
-      <c r="L234" t="inlineStr"/>
       <c r="M234" t="n">
         <v>1</v>
       </c>
@@ -8665,10 +7733,6 @@
       <c r="H235" t="n">
         <v>2</v>
       </c>
-      <c r="I235" t="inlineStr"/>
-      <c r="J235" t="inlineStr"/>
-      <c r="K235" t="inlineStr"/>
-      <c r="L235" t="inlineStr"/>
       <c r="M235" t="n">
         <v>1</v>
       </c>
@@ -8700,10 +7764,6 @@
       <c r="H236" t="n">
         <v>2</v>
       </c>
-      <c r="I236" t="inlineStr"/>
-      <c r="J236" t="inlineStr"/>
-      <c r="K236" t="inlineStr"/>
-      <c r="L236" t="inlineStr"/>
       <c r="M236" t="n">
         <v>1</v>
       </c>
@@ -8735,10 +7795,6 @@
       <c r="H237" t="n">
         <v>2</v>
       </c>
-      <c r="I237" t="inlineStr"/>
-      <c r="J237" t="inlineStr"/>
-      <c r="K237" t="inlineStr"/>
-      <c r="L237" t="inlineStr"/>
       <c r="M237" t="n">
         <v>1</v>
       </c>
@@ -8770,10 +7826,6 @@
       <c r="H238" t="n">
         <v>2</v>
       </c>
-      <c r="I238" t="inlineStr"/>
-      <c r="J238" t="inlineStr"/>
-      <c r="K238" t="inlineStr"/>
-      <c r="L238" t="inlineStr"/>
       <c r="M238" t="n">
         <v>1</v>
       </c>
@@ -8805,10 +7857,6 @@
       <c r="H239" t="n">
         <v>2</v>
       </c>
-      <c r="I239" t="inlineStr"/>
-      <c r="J239" t="inlineStr"/>
-      <c r="K239" t="inlineStr"/>
-      <c r="L239" t="inlineStr"/>
       <c r="M239" t="n">
         <v>1</v>
       </c>
@@ -8840,10 +7888,6 @@
       <c r="H240" t="n">
         <v>2</v>
       </c>
-      <c r="I240" t="inlineStr"/>
-      <c r="J240" t="inlineStr"/>
-      <c r="K240" t="inlineStr"/>
-      <c r="L240" t="inlineStr"/>
       <c r="M240" t="n">
         <v>1</v>
       </c>
@@ -8875,10 +7919,6 @@
       <c r="H241" t="n">
         <v>2</v>
       </c>
-      <c r="I241" t="inlineStr"/>
-      <c r="J241" t="inlineStr"/>
-      <c r="K241" t="inlineStr"/>
-      <c r="L241" t="inlineStr"/>
       <c r="M241" t="n">
         <v>1</v>
       </c>
@@ -8910,10 +7950,6 @@
       <c r="H242" t="n">
         <v>2</v>
       </c>
-      <c r="I242" t="inlineStr"/>
-      <c r="J242" t="inlineStr"/>
-      <c r="K242" t="inlineStr"/>
-      <c r="L242" t="inlineStr"/>
       <c r="M242" t="n">
         <v>1</v>
       </c>
@@ -8945,10 +7981,6 @@
       <c r="H243" t="n">
         <v>2</v>
       </c>
-      <c r="I243" t="inlineStr"/>
-      <c r="J243" t="inlineStr"/>
-      <c r="K243" t="inlineStr"/>
-      <c r="L243" t="inlineStr"/>
       <c r="M243" t="n">
         <v>1</v>
       </c>
@@ -8962,7 +7994,7 @@
       </c>
       <c r="C244" t="inlineStr">
         <is>
-          <t>Prepaid items</t>
+          <t>Prepaid Items</t>
         </is>
       </c>
       <c r="D244" t="n">
@@ -8980,10 +8012,6 @@
       <c r="H244" t="n">
         <v>2</v>
       </c>
-      <c r="I244" t="inlineStr"/>
-      <c r="J244" t="inlineStr"/>
-      <c r="K244" t="inlineStr"/>
-      <c r="L244" t="inlineStr"/>
       <c r="M244" t="n">
         <v>1</v>
       </c>
@@ -9015,10 +8043,6 @@
       <c r="H245" t="n">
         <v>2</v>
       </c>
-      <c r="I245" t="inlineStr"/>
-      <c r="J245" t="inlineStr"/>
-      <c r="K245" t="inlineStr"/>
-      <c r="L245" t="inlineStr"/>
       <c r="M245" t="n">
         <v>1</v>
       </c>
@@ -9050,10 +8074,6 @@
       <c r="H246" t="n">
         <v>2</v>
       </c>
-      <c r="I246" t="inlineStr"/>
-      <c r="J246" t="inlineStr"/>
-      <c r="K246" t="inlineStr"/>
-      <c r="L246" t="inlineStr"/>
       <c r="M246" t="n">
         <v>1</v>
       </c>
@@ -9085,10 +8105,6 @@
       <c r="H247" t="n">
         <v>2</v>
       </c>
-      <c r="I247" t="inlineStr"/>
-      <c r="J247" t="inlineStr"/>
-      <c r="K247" t="inlineStr"/>
-      <c r="L247" t="inlineStr"/>
       <c r="M247" t="n">
         <v>1</v>
       </c>
@@ -9120,10 +8136,6 @@
       <c r="H248" t="n">
         <v>2</v>
       </c>
-      <c r="I248" t="inlineStr"/>
-      <c r="J248" t="inlineStr"/>
-      <c r="K248" t="inlineStr"/>
-      <c r="L248" t="inlineStr"/>
       <c r="M248" t="n">
         <v>1</v>
       </c>
@@ -9155,10 +8167,6 @@
       <c r="H249" t="n">
         <v>2</v>
       </c>
-      <c r="I249" t="inlineStr"/>
-      <c r="J249" t="inlineStr"/>
-      <c r="K249" t="inlineStr"/>
-      <c r="L249" t="inlineStr"/>
       <c r="M249" t="n">
         <v>1</v>
       </c>
@@ -9190,10 +8198,6 @@
       <c r="H250" t="n">
         <v>2</v>
       </c>
-      <c r="I250" t="inlineStr"/>
-      <c r="J250" t="inlineStr"/>
-      <c r="K250" t="inlineStr"/>
-      <c r="L250" t="inlineStr"/>
       <c r="M250" t="n">
         <v>1</v>
       </c>
@@ -9225,10 +8229,6 @@
       <c r="H251" t="n">
         <v>2</v>
       </c>
-      <c r="I251" t="inlineStr"/>
-      <c r="J251" t="inlineStr"/>
-      <c r="K251" t="inlineStr"/>
-      <c r="L251" t="inlineStr"/>
       <c r="M251" t="n">
         <v>1</v>
       </c>
@@ -9260,10 +8260,6 @@
       <c r="H252" t="n">
         <v>3</v>
       </c>
-      <c r="I252" t="inlineStr"/>
-      <c r="J252" t="inlineStr"/>
-      <c r="K252" t="inlineStr"/>
-      <c r="L252" t="inlineStr"/>
       <c r="M252" t="n">
         <v>1</v>
       </c>
@@ -9295,10 +8291,6 @@
       <c r="H253" t="n">
         <v>3</v>
       </c>
-      <c r="I253" t="inlineStr"/>
-      <c r="J253" t="inlineStr"/>
-      <c r="K253" t="inlineStr"/>
-      <c r="L253" t="inlineStr"/>
       <c r="M253" t="n">
         <v>1</v>
       </c>
@@ -9330,10 +8322,6 @@
       <c r="H254" t="n">
         <v>3</v>
       </c>
-      <c r="I254" t="inlineStr"/>
-      <c r="J254" t="inlineStr"/>
-      <c r="K254" t="inlineStr"/>
-      <c r="L254" t="inlineStr"/>
       <c r="M254" t="n">
         <v>1</v>
       </c>
@@ -9365,10 +8353,6 @@
       <c r="H255" t="n">
         <v>3</v>
       </c>
-      <c r="I255" t="inlineStr"/>
-      <c r="J255" t="inlineStr"/>
-      <c r="K255" t="inlineStr"/>
-      <c r="L255" t="inlineStr"/>
       <c r="M255" t="n">
         <v>1</v>
       </c>
@@ -9400,10 +8384,6 @@
       <c r="H256" t="n">
         <v>3</v>
       </c>
-      <c r="I256" t="inlineStr"/>
-      <c r="J256" t="inlineStr"/>
-      <c r="K256" t="inlineStr"/>
-      <c r="L256" t="inlineStr"/>
       <c r="M256" t="n">
         <v>1</v>
       </c>
@@ -9435,10 +8415,6 @@
       <c r="H257" t="n">
         <v>3</v>
       </c>
-      <c r="I257" t="inlineStr"/>
-      <c r="J257" t="inlineStr"/>
-      <c r="K257" t="inlineStr"/>
-      <c r="L257" t="inlineStr"/>
       <c r="M257" t="n">
         <v>1</v>
       </c>
@@ -9470,10 +8446,6 @@
       <c r="H258" t="n">
         <v>3</v>
       </c>
-      <c r="I258" t="inlineStr"/>
-      <c r="J258" t="inlineStr"/>
-      <c r="K258" t="inlineStr"/>
-      <c r="L258" t="inlineStr"/>
       <c r="M258" t="n">
         <v>1</v>
       </c>
@@ -9505,10 +8477,6 @@
       <c r="H259" t="n">
         <v>3</v>
       </c>
-      <c r="I259" t="inlineStr"/>
-      <c r="J259" t="inlineStr"/>
-      <c r="K259" t="inlineStr"/>
-      <c r="L259" t="inlineStr"/>
       <c r="M259" t="n">
         <v>1</v>
       </c>
@@ -9540,10 +8508,6 @@
       <c r="H260" t="n">
         <v>3</v>
       </c>
-      <c r="I260" t="inlineStr"/>
-      <c r="J260" t="inlineStr"/>
-      <c r="K260" t="inlineStr"/>
-      <c r="L260" t="inlineStr"/>
       <c r="M260" t="n">
         <v>1</v>
       </c>
@@ -9575,10 +8539,6 @@
       <c r="H261" t="n">
         <v>1</v>
       </c>
-      <c r="I261" t="inlineStr"/>
-      <c r="J261" t="inlineStr"/>
-      <c r="K261" t="inlineStr"/>
-      <c r="L261" t="inlineStr"/>
       <c r="M261" t="n">
         <v>1</v>
       </c>
@@ -9610,10 +8570,6 @@
       <c r="H262" t="n">
         <v>2</v>
       </c>
-      <c r="I262" t="inlineStr"/>
-      <c r="J262" t="inlineStr"/>
-      <c r="K262" t="inlineStr"/>
-      <c r="L262" t="inlineStr"/>
       <c r="M262" t="n">
         <v>1</v>
       </c>
@@ -9645,10 +8601,6 @@
       <c r="H263" t="n">
         <v>3</v>
       </c>
-      <c r="I263" t="inlineStr"/>
-      <c r="J263" t="inlineStr"/>
-      <c r="K263" t="inlineStr"/>
-      <c r="L263" t="inlineStr"/>
       <c r="M263" t="n">
         <v>1</v>
       </c>
@@ -9680,10 +8632,6 @@
       <c r="H264" t="n">
         <v>3</v>
       </c>
-      <c r="I264" t="inlineStr"/>
-      <c r="J264" t="inlineStr"/>
-      <c r="K264" t="inlineStr"/>
-      <c r="L264" t="inlineStr"/>
       <c r="M264" t="n">
         <v>1</v>
       </c>
@@ -9715,10 +8663,6 @@
       <c r="H265" t="n">
         <v>1</v>
       </c>
-      <c r="I265" t="inlineStr"/>
-      <c r="J265" t="inlineStr"/>
-      <c r="K265" t="inlineStr"/>
-      <c r="L265" t="inlineStr"/>
       <c r="M265" t="n">
         <v>1</v>
       </c>
@@ -9750,10 +8694,6 @@
       <c r="H266" t="n">
         <v>2</v>
       </c>
-      <c r="I266" t="inlineStr"/>
-      <c r="J266" t="inlineStr"/>
-      <c r="K266" t="inlineStr"/>
-      <c r="L266" t="inlineStr"/>
       <c r="M266" t="n">
         <v>1</v>
       </c>
@@ -9785,10 +8725,6 @@
       <c r="H267" t="n">
         <v>2</v>
       </c>
-      <c r="I267" t="inlineStr"/>
-      <c r="J267" t="inlineStr"/>
-      <c r="K267" t="inlineStr"/>
-      <c r="L267" t="inlineStr"/>
       <c r="M267" t="n">
         <v>1</v>
       </c>
@@ -9820,10 +8756,6 @@
       <c r="H268" t="n">
         <v>2</v>
       </c>
-      <c r="I268" t="inlineStr"/>
-      <c r="J268" t="inlineStr"/>
-      <c r="K268" t="inlineStr"/>
-      <c r="L268" t="inlineStr"/>
       <c r="M268" t="n">
         <v>1</v>
       </c>
@@ -9855,10 +8787,6 @@
       <c r="H269" t="n">
         <v>2</v>
       </c>
-      <c r="I269" t="inlineStr"/>
-      <c r="J269" t="inlineStr"/>
-      <c r="K269" t="inlineStr"/>
-      <c r="L269" t="inlineStr"/>
       <c r="M269" t="n">
         <v>1</v>
       </c>
@@ -9890,10 +8818,6 @@
       <c r="H270" t="n">
         <v>2</v>
       </c>
-      <c r="I270" t="inlineStr"/>
-      <c r="J270" t="inlineStr"/>
-      <c r="K270" t="inlineStr"/>
-      <c r="L270" t="inlineStr"/>
       <c r="M270" t="n">
         <v>1</v>
       </c>
@@ -9925,10 +8849,6 @@
       <c r="H271" t="n">
         <v>2</v>
       </c>
-      <c r="I271" t="inlineStr"/>
-      <c r="J271" t="inlineStr"/>
-      <c r="K271" t="inlineStr"/>
-      <c r="L271" t="inlineStr"/>
       <c r="M271" t="n">
         <v>1</v>
       </c>
@@ -9960,10 +8880,6 @@
       <c r="H272" t="n">
         <v>2</v>
       </c>
-      <c r="I272" t="inlineStr"/>
-      <c r="J272" t="inlineStr"/>
-      <c r="K272" t="inlineStr"/>
-      <c r="L272" t="inlineStr"/>
       <c r="M272" t="n">
         <v>1</v>
       </c>
@@ -9995,10 +8911,6 @@
       <c r="H273" t="n">
         <v>2</v>
       </c>
-      <c r="I273" t="inlineStr"/>
-      <c r="J273" t="inlineStr"/>
-      <c r="K273" t="inlineStr"/>
-      <c r="L273" t="inlineStr"/>
       <c r="M273" t="n">
         <v>1</v>
       </c>
@@ -10030,10 +8942,6 @@
       <c r="H274" t="n">
         <v>2</v>
       </c>
-      <c r="I274" t="inlineStr"/>
-      <c r="J274" t="inlineStr"/>
-      <c r="K274" t="inlineStr"/>
-      <c r="L274" t="inlineStr"/>
       <c r="M274" t="n">
         <v>1</v>
       </c>
@@ -10065,10 +8973,6 @@
       <c r="H275" t="n">
         <v>2</v>
       </c>
-      <c r="I275" t="inlineStr"/>
-      <c r="J275" t="inlineStr"/>
-      <c r="K275" t="inlineStr"/>
-      <c r="L275" t="inlineStr"/>
       <c r="M275" t="n">
         <v>1</v>
       </c>
@@ -10100,10 +9004,6 @@
       <c r="H276" t="n">
         <v>2</v>
       </c>
-      <c r="I276" t="inlineStr"/>
-      <c r="J276" t="inlineStr"/>
-      <c r="K276" t="inlineStr"/>
-      <c r="L276" t="inlineStr"/>
       <c r="M276" t="n">
         <v>1</v>
       </c>
@@ -10135,10 +9035,6 @@
       <c r="H277" t="n">
         <v>2</v>
       </c>
-      <c r="I277" t="inlineStr"/>
-      <c r="J277" t="inlineStr"/>
-      <c r="K277" t="inlineStr"/>
-      <c r="L277" t="inlineStr"/>
       <c r="M277" t="n">
         <v>1</v>
       </c>
@@ -10170,10 +9066,6 @@
       <c r="H278" t="n">
         <v>2</v>
       </c>
-      <c r="I278" t="inlineStr"/>
-      <c r="J278" t="inlineStr"/>
-      <c r="K278" t="inlineStr"/>
-      <c r="L278" t="inlineStr"/>
       <c r="M278" t="n">
         <v>1</v>
       </c>
@@ -10205,10 +9097,6 @@
       <c r="H279" t="n">
         <v>2</v>
       </c>
-      <c r="I279" t="inlineStr"/>
-      <c r="J279" t="inlineStr"/>
-      <c r="K279" t="inlineStr"/>
-      <c r="L279" t="inlineStr"/>
       <c r="M279" t="n">
         <v>1</v>
       </c>
@@ -10240,10 +9128,6 @@
       <c r="H280" t="n">
         <v>2</v>
       </c>
-      <c r="I280" t="inlineStr"/>
-      <c r="J280" t="inlineStr"/>
-      <c r="K280" t="inlineStr"/>
-      <c r="L280" t="inlineStr"/>
       <c r="M280" t="n">
         <v>1</v>
       </c>
@@ -10275,10 +9159,6 @@
       <c r="H281" t="n">
         <v>2</v>
       </c>
-      <c r="I281" t="inlineStr"/>
-      <c r="J281" t="inlineStr"/>
-      <c r="K281" t="inlineStr"/>
-      <c r="L281" t="inlineStr"/>
       <c r="M281" t="n">
         <v>1</v>
       </c>
@@ -10310,10 +9190,6 @@
       <c r="H282" t="n">
         <v>2</v>
       </c>
-      <c r="I282" t="inlineStr"/>
-      <c r="J282" t="inlineStr"/>
-      <c r="K282" t="inlineStr"/>
-      <c r="L282" t="inlineStr"/>
       <c r="M282" t="n">
         <v>1</v>
       </c>
@@ -10345,10 +9221,6 @@
       <c r="H283" t="n">
         <v>3</v>
       </c>
-      <c r="I283" t="inlineStr"/>
-      <c r="J283" t="inlineStr"/>
-      <c r="K283" t="inlineStr"/>
-      <c r="L283" t="inlineStr"/>
       <c r="M283" t="n">
         <v>1</v>
       </c>
@@ -10380,10 +9252,6 @@
       <c r="H284" t="n">
         <v>3</v>
       </c>
-      <c r="I284" t="inlineStr"/>
-      <c r="J284" t="inlineStr"/>
-      <c r="K284" t="inlineStr"/>
-      <c r="L284" t="inlineStr"/>
       <c r="M284" t="n">
         <v>1</v>
       </c>
@@ -10415,10 +9283,6 @@
       <c r="H285" t="n">
         <v>3</v>
       </c>
-      <c r="I285" t="inlineStr"/>
-      <c r="J285" t="inlineStr"/>
-      <c r="K285" t="inlineStr"/>
-      <c r="L285" t="inlineStr"/>
       <c r="M285" t="n">
         <v>1</v>
       </c>
@@ -10450,10 +9314,6 @@
       <c r="H286" t="n">
         <v>1</v>
       </c>
-      <c r="I286" t="inlineStr"/>
-      <c r="J286" t="inlineStr"/>
-      <c r="K286" t="inlineStr"/>
-      <c r="L286" t="inlineStr"/>
       <c r="M286" t="n">
         <v>1</v>
       </c>
@@ -10485,10 +9345,6 @@
       <c r="H287" t="n">
         <v>2</v>
       </c>
-      <c r="I287" t="inlineStr"/>
-      <c r="J287" t="inlineStr"/>
-      <c r="K287" t="inlineStr"/>
-      <c r="L287" t="inlineStr"/>
       <c r="M287" t="n">
         <v>1</v>
       </c>
@@ -10520,10 +9376,6 @@
       <c r="H288" t="n">
         <v>3</v>
       </c>
-      <c r="I288" t="inlineStr"/>
-      <c r="J288" t="inlineStr"/>
-      <c r="K288" t="inlineStr"/>
-      <c r="L288" t="inlineStr"/>
       <c r="M288" t="n">
         <v>1</v>
       </c>
@@ -10555,10 +9407,6 @@
       <c r="H289" t="n">
         <v>3</v>
       </c>
-      <c r="I289" t="inlineStr"/>
-      <c r="J289" t="inlineStr"/>
-      <c r="K289" t="inlineStr"/>
-      <c r="L289" t="inlineStr"/>
       <c r="M289" t="n">
         <v>1</v>
       </c>
@@ -10590,10 +9438,6 @@
       <c r="H290" t="n">
         <v>1</v>
       </c>
-      <c r="I290" t="inlineStr"/>
-      <c r="J290" t="inlineStr"/>
-      <c r="K290" t="inlineStr"/>
-      <c r="L290" t="inlineStr"/>
       <c r="M290" t="n">
         <v>1</v>
       </c>
@@ -10625,10 +9469,6 @@
       <c r="H291" t="n">
         <v>2</v>
       </c>
-      <c r="I291" t="inlineStr"/>
-      <c r="J291" t="inlineStr"/>
-      <c r="K291" t="inlineStr"/>
-      <c r="L291" t="inlineStr"/>
       <c r="M291" t="n">
         <v>1</v>
       </c>
@@ -10660,10 +9500,6 @@
       <c r="H292" t="n">
         <v>2</v>
       </c>
-      <c r="I292" t="inlineStr"/>
-      <c r="J292" t="inlineStr"/>
-      <c r="K292" t="inlineStr"/>
-      <c r="L292" t="inlineStr"/>
       <c r="M292" t="n">
         <v>1</v>
       </c>
@@ -10695,10 +9531,6 @@
       <c r="H293" t="n">
         <v>2</v>
       </c>
-      <c r="I293" t="inlineStr"/>
-      <c r="J293" t="inlineStr"/>
-      <c r="K293" t="inlineStr"/>
-      <c r="L293" t="inlineStr"/>
       <c r="M293" t="n">
         <v>1</v>
       </c>
@@ -10730,10 +9562,6 @@
       <c r="H294" t="n">
         <v>3</v>
       </c>
-      <c r="I294" t="inlineStr"/>
-      <c r="J294" t="inlineStr"/>
-      <c r="K294" t="inlineStr"/>
-      <c r="L294" t="inlineStr"/>
       <c r="M294" t="n">
         <v>1</v>
       </c>
@@ -10765,10 +9593,6 @@
       <c r="H295" t="n">
         <v>3</v>
       </c>
-      <c r="I295" t="inlineStr"/>
-      <c r="J295" t="inlineStr"/>
-      <c r="K295" t="inlineStr"/>
-      <c r="L295" t="inlineStr"/>
       <c r="M295" t="n">
         <v>1</v>
       </c>
@@ -10800,10 +9624,6 @@
       <c r="H296" t="n">
         <v>3</v>
       </c>
-      <c r="I296" t="inlineStr"/>
-      <c r="J296" t="inlineStr"/>
-      <c r="K296" t="inlineStr"/>
-      <c r="L296" t="inlineStr"/>
       <c r="M296" t="n">
         <v>1</v>
       </c>
@@ -10835,10 +9655,6 @@
       <c r="H297" t="n">
         <v>3</v>
       </c>
-      <c r="I297" t="inlineStr"/>
-      <c r="J297" t="inlineStr"/>
-      <c r="K297" t="inlineStr"/>
-      <c r="L297" t="inlineStr"/>
       <c r="M297" t="n">
         <v>1</v>
       </c>
@@ -10852,7 +9668,7 @@
       </c>
       <c r="C298" t="inlineStr">
         <is>
-          <t>Total Liabilities, Deferred inflows of resources, and Net position</t>
+          <t>Total Liabilities, Deferred Inflows of Resources, and Net Position</t>
         </is>
       </c>
       <c r="D298" t="n">
@@ -10870,10 +9686,6 @@
       <c r="H298" t="n">
         <v>3</v>
       </c>
-      <c r="I298" t="inlineStr"/>
-      <c r="J298" t="inlineStr"/>
-      <c r="K298" t="inlineStr"/>
-      <c r="L298" t="inlineStr"/>
       <c r="M298" t="n">
         <v>1</v>
       </c>
@@ -10905,10 +9717,6 @@
       <c r="H299" t="n">
         <v>2</v>
       </c>
-      <c r="I299" t="inlineStr"/>
-      <c r="J299" t="inlineStr"/>
-      <c r="K299" t="inlineStr"/>
-      <c r="L299" t="inlineStr"/>
       <c r="M299" t="n">
         <v>1</v>
       </c>
@@ -10940,10 +9748,6 @@
       <c r="H300" t="n">
         <v>1</v>
       </c>
-      <c r="I300" t="inlineStr"/>
-      <c r="J300" t="inlineStr"/>
-      <c r="K300" t="inlineStr"/>
-      <c r="L300" t="inlineStr"/>
       <c r="M300" t="n">
         <v>1</v>
       </c>
@@ -10975,10 +9779,6 @@
       <c r="H301" t="n">
         <v>2</v>
       </c>
-      <c r="I301" t="inlineStr"/>
-      <c r="J301" t="inlineStr"/>
-      <c r="K301" t="inlineStr"/>
-      <c r="L301" t="inlineStr"/>
       <c r="M301" t="n">
         <v>1</v>
       </c>
@@ -11010,10 +9810,6 @@
       <c r="H302" t="n">
         <v>2</v>
       </c>
-      <c r="I302" t="inlineStr"/>
-      <c r="J302" t="inlineStr"/>
-      <c r="K302" t="inlineStr"/>
-      <c r="L302" t="inlineStr"/>
       <c r="M302" t="n">
         <v>1</v>
       </c>
@@ -11045,10 +9841,6 @@
       <c r="H303" t="n">
         <v>2</v>
       </c>
-      <c r="I303" t="inlineStr"/>
-      <c r="J303" t="inlineStr"/>
-      <c r="K303" t="inlineStr"/>
-      <c r="L303" t="inlineStr"/>
       <c r="M303" t="n">
         <v>1</v>
       </c>
@@ -11080,10 +9872,6 @@
       <c r="H304" t="n">
         <v>2</v>
       </c>
-      <c r="I304" t="inlineStr"/>
-      <c r="J304" t="inlineStr"/>
-      <c r="K304" t="inlineStr"/>
-      <c r="L304" t="inlineStr"/>
       <c r="M304" t="n">
         <v>1</v>
       </c>
@@ -11115,10 +9903,6 @@
       <c r="H305" t="n">
         <v>2</v>
       </c>
-      <c r="I305" t="inlineStr"/>
-      <c r="J305" t="inlineStr"/>
-      <c r="K305" t="inlineStr"/>
-      <c r="L305" t="inlineStr"/>
       <c r="M305" t="n">
         <v>1</v>
       </c>
@@ -11150,10 +9934,6 @@
       <c r="H306" t="n">
         <v>3</v>
       </c>
-      <c r="I306" t="inlineStr"/>
-      <c r="J306" t="inlineStr"/>
-      <c r="K306" t="inlineStr"/>
-      <c r="L306" t="inlineStr"/>
       <c r="M306" t="n">
         <v>1</v>
       </c>
@@ -11185,10 +9965,6 @@
       <c r="H307" t="n">
         <v>3</v>
       </c>
-      <c r="I307" t="inlineStr"/>
-      <c r="J307" t="inlineStr"/>
-      <c r="K307" t="inlineStr"/>
-      <c r="L307" t="inlineStr"/>
       <c r="M307" t="n">
         <v>1</v>
       </c>
@@ -11220,10 +9996,6 @@
       <c r="H308" t="n">
         <v>3</v>
       </c>
-      <c r="I308" t="inlineStr"/>
-      <c r="J308" t="inlineStr"/>
-      <c r="K308" t="inlineStr"/>
-      <c r="L308" t="inlineStr"/>
       <c r="M308" t="n">
         <v>1</v>
       </c>
@@ -11255,10 +10027,6 @@
       <c r="H309" t="n">
         <v>1</v>
       </c>
-      <c r="I309" t="inlineStr"/>
-      <c r="J309" t="inlineStr"/>
-      <c r="K309" t="inlineStr"/>
-      <c r="L309" t="inlineStr"/>
       <c r="M309" t="n">
         <v>1</v>
       </c>
@@ -11290,10 +10058,6 @@
       <c r="H310" t="n">
         <v>2</v>
       </c>
-      <c r="I310" t="inlineStr"/>
-      <c r="J310" t="inlineStr"/>
-      <c r="K310" t="inlineStr"/>
-      <c r="L310" t="inlineStr"/>
       <c r="M310" t="n">
         <v>1</v>
       </c>
@@ -11325,10 +10089,6 @@
       <c r="H311" t="n">
         <v>2</v>
       </c>
-      <c r="I311" t="inlineStr"/>
-      <c r="J311" t="inlineStr"/>
-      <c r="K311" t="inlineStr"/>
-      <c r="L311" t="inlineStr"/>
       <c r="M311" t="n">
         <v>1</v>
       </c>
@@ -11360,10 +10120,6 @@
       <c r="H312" t="n">
         <v>2</v>
       </c>
-      <c r="I312" t="inlineStr"/>
-      <c r="J312" t="inlineStr"/>
-      <c r="K312" t="inlineStr"/>
-      <c r="L312" t="inlineStr"/>
       <c r="M312" t="n">
         <v>1</v>
       </c>
@@ -11395,10 +10151,6 @@
       <c r="H313" t="n">
         <v>2</v>
       </c>
-      <c r="I313" t="inlineStr"/>
-      <c r="J313" t="inlineStr"/>
-      <c r="K313" t="inlineStr"/>
-      <c r="L313" t="inlineStr"/>
       <c r="M313" t="n">
         <v>1</v>
       </c>
@@ -11430,10 +10182,6 @@
       <c r="H314" t="n">
         <v>2</v>
       </c>
-      <c r="I314" t="inlineStr"/>
-      <c r="J314" t="inlineStr"/>
-      <c r="K314" t="inlineStr"/>
-      <c r="L314" t="inlineStr"/>
       <c r="M314" t="n">
         <v>1</v>
       </c>
@@ -11465,10 +10213,6 @@
       <c r="H315" t="n">
         <v>2</v>
       </c>
-      <c r="I315" t="inlineStr"/>
-      <c r="J315" t="inlineStr"/>
-      <c r="K315" t="inlineStr"/>
-      <c r="L315" t="inlineStr"/>
       <c r="M315" t="n">
         <v>1</v>
       </c>
@@ -11500,10 +10244,6 @@
       <c r="H316" t="n">
         <v>2</v>
       </c>
-      <c r="I316" t="inlineStr"/>
-      <c r="J316" t="inlineStr"/>
-      <c r="K316" t="inlineStr"/>
-      <c r="L316" t="inlineStr"/>
       <c r="M316" t="n">
         <v>1</v>
       </c>
@@ -11535,10 +10275,6 @@
       <c r="H317" t="n">
         <v>2</v>
       </c>
-      <c r="I317" t="inlineStr"/>
-      <c r="J317" t="inlineStr"/>
-      <c r="K317" t="inlineStr"/>
-      <c r="L317" t="inlineStr"/>
       <c r="M317" t="n">
         <v>1</v>
       </c>
@@ -11570,10 +10306,6 @@
       <c r="H318" t="n">
         <v>2</v>
       </c>
-      <c r="I318" t="inlineStr"/>
-      <c r="J318" t="inlineStr"/>
-      <c r="K318" t="inlineStr"/>
-      <c r="L318" t="inlineStr"/>
       <c r="M318" t="n">
         <v>1</v>
       </c>
@@ -11605,10 +10337,6 @@
       <c r="H319" t="n">
         <v>3</v>
       </c>
-      <c r="I319" t="inlineStr"/>
-      <c r="J319" t="inlineStr"/>
-      <c r="K319" t="inlineStr"/>
-      <c r="L319" t="inlineStr"/>
       <c r="M319" t="n">
         <v>1</v>
       </c>
@@ -11640,10 +10368,6 @@
       <c r="H320" t="n">
         <v>1</v>
       </c>
-      <c r="I320" t="inlineStr"/>
-      <c r="J320" t="inlineStr"/>
-      <c r="K320" t="inlineStr"/>
-      <c r="L320" t="inlineStr"/>
       <c r="M320" t="n">
         <v>1</v>
       </c>
@@ -11675,10 +10399,6 @@
       <c r="H321" t="n">
         <v>2</v>
       </c>
-      <c r="I321" t="inlineStr"/>
-      <c r="J321" t="inlineStr"/>
-      <c r="K321" t="inlineStr"/>
-      <c r="L321" t="inlineStr"/>
       <c r="M321" t="n">
         <v>1</v>
       </c>
@@ -11710,10 +10430,6 @@
       <c r="H322" t="n">
         <v>2</v>
       </c>
-      <c r="I322" t="inlineStr"/>
-      <c r="J322" t="inlineStr"/>
-      <c r="K322" t="inlineStr"/>
-      <c r="L322" t="inlineStr"/>
       <c r="M322" t="n">
         <v>1</v>
       </c>
@@ -11745,10 +10461,6 @@
       <c r="H323" t="n">
         <v>2</v>
       </c>
-      <c r="I323" t="inlineStr"/>
-      <c r="J323" t="inlineStr"/>
-      <c r="K323" t="inlineStr"/>
-      <c r="L323" t="inlineStr"/>
       <c r="M323" t="n">
         <v>1</v>
       </c>
@@ -11780,10 +10492,6 @@
       <c r="H324" t="n">
         <v>2</v>
       </c>
-      <c r="I324" t="inlineStr"/>
-      <c r="J324" t="inlineStr"/>
-      <c r="K324" t="inlineStr"/>
-      <c r="L324" t="inlineStr"/>
       <c r="M324" t="n">
         <v>1</v>
       </c>
@@ -11815,10 +10523,6 @@
       <c r="H325" t="n">
         <v>2</v>
       </c>
-      <c r="I325" t="inlineStr"/>
-      <c r="J325" t="inlineStr"/>
-      <c r="K325" t="inlineStr"/>
-      <c r="L325" t="inlineStr"/>
       <c r="M325" t="n">
         <v>1</v>
       </c>
@@ -11850,10 +10554,6 @@
       <c r="H326" t="n">
         <v>2</v>
       </c>
-      <c r="I326" t="inlineStr"/>
-      <c r="J326" t="inlineStr"/>
-      <c r="K326" t="inlineStr"/>
-      <c r="L326" t="inlineStr"/>
       <c r="M326" t="n">
         <v>1</v>
       </c>
@@ -11885,10 +10585,6 @@
       <c r="H327" t="n">
         <v>2</v>
       </c>
-      <c r="I327" t="inlineStr"/>
-      <c r="J327" t="inlineStr"/>
-      <c r="K327" t="inlineStr"/>
-      <c r="L327" t="inlineStr"/>
       <c r="M327" t="n">
         <v>1</v>
       </c>
@@ -11920,10 +10616,6 @@
       <c r="H328" t="n">
         <v>2</v>
       </c>
-      <c r="I328" t="inlineStr"/>
-      <c r="J328" t="inlineStr"/>
-      <c r="K328" t="inlineStr"/>
-      <c r="L328" t="inlineStr"/>
       <c r="M328" t="n">
         <v>1</v>
       </c>
@@ -11955,10 +10647,6 @@
       <c r="H329" t="n">
         <v>2</v>
       </c>
-      <c r="I329" t="inlineStr"/>
-      <c r="J329" t="inlineStr"/>
-      <c r="K329" t="inlineStr"/>
-      <c r="L329" t="inlineStr"/>
       <c r="M329" t="n">
         <v>1</v>
       </c>
@@ -11990,10 +10678,6 @@
       <c r="H330" t="n">
         <v>2</v>
       </c>
-      <c r="I330" t="inlineStr"/>
-      <c r="J330" t="inlineStr"/>
-      <c r="K330" t="inlineStr"/>
-      <c r="L330" t="inlineStr"/>
       <c r="M330" t="n">
         <v>1</v>
       </c>
@@ -12025,10 +10709,6 @@
       <c r="H331" t="n">
         <v>3</v>
       </c>
-      <c r="I331" t="inlineStr"/>
-      <c r="J331" t="inlineStr"/>
-      <c r="K331" t="inlineStr"/>
-      <c r="L331" t="inlineStr"/>
       <c r="M331" t="n">
         <v>1</v>
       </c>
@@ -12060,10 +10740,6 @@
       <c r="H332" t="n">
         <v>3</v>
       </c>
-      <c r="I332" t="inlineStr"/>
-      <c r="J332" t="inlineStr"/>
-      <c r="K332" t="inlineStr"/>
-      <c r="L332" t="inlineStr"/>
       <c r="M332" t="n">
         <v>1</v>
       </c>
@@ -12095,10 +10771,6 @@
       <c r="H333" t="n">
         <v>1</v>
       </c>
-      <c r="I333" t="inlineStr"/>
-      <c r="J333" t="inlineStr"/>
-      <c r="K333" t="inlineStr"/>
-      <c r="L333" t="inlineStr"/>
       <c r="M333" t="n">
         <v>1</v>
       </c>
@@ -12130,10 +10802,6 @@
       <c r="H334" t="n">
         <v>2</v>
       </c>
-      <c r="I334" t="inlineStr"/>
-      <c r="J334" t="inlineStr"/>
-      <c r="K334" t="inlineStr"/>
-      <c r="L334" t="inlineStr"/>
       <c r="M334" t="n">
         <v>1</v>
       </c>
@@ -12165,10 +10833,6 @@
       <c r="H335" t="n">
         <v>2</v>
       </c>
-      <c r="I335" t="inlineStr"/>
-      <c r="J335" t="inlineStr"/>
-      <c r="K335" t="inlineStr"/>
-      <c r="L335" t="inlineStr"/>
       <c r="M335" t="n">
         <v>1</v>
       </c>
@@ -12200,10 +10864,6 @@
       <c r="H336" t="n">
         <v>2</v>
       </c>
-      <c r="I336" t="inlineStr"/>
-      <c r="J336" t="inlineStr"/>
-      <c r="K336" t="inlineStr"/>
-      <c r="L336" t="inlineStr"/>
       <c r="M336" t="n">
         <v>1</v>
       </c>
@@ -12235,10 +10895,6 @@
       <c r="H337" t="n">
         <v>2</v>
       </c>
-      <c r="I337" t="inlineStr"/>
-      <c r="J337" t="inlineStr"/>
-      <c r="K337" t="inlineStr"/>
-      <c r="L337" t="inlineStr"/>
       <c r="M337" t="n">
         <v>1</v>
       </c>
@@ -12270,10 +10926,6 @@
       <c r="H338" t="n">
         <v>2</v>
       </c>
-      <c r="I338" t="inlineStr"/>
-      <c r="J338" t="inlineStr"/>
-      <c r="K338" t="inlineStr"/>
-      <c r="L338" t="inlineStr"/>
       <c r="M338" t="n">
         <v>1</v>
       </c>
@@ -12305,10 +10957,6 @@
       <c r="H339" t="n">
         <v>2</v>
       </c>
-      <c r="I339" t="inlineStr"/>
-      <c r="J339" t="inlineStr"/>
-      <c r="K339" t="inlineStr"/>
-      <c r="L339" t="inlineStr"/>
       <c r="M339" t="n">
         <v>1</v>
       </c>
@@ -12340,10 +10988,6 @@
       <c r="H340" t="n">
         <v>2</v>
       </c>
-      <c r="I340" t="inlineStr"/>
-      <c r="J340" t="inlineStr"/>
-      <c r="K340" t="inlineStr"/>
-      <c r="L340" t="inlineStr"/>
       <c r="M340" t="n">
         <v>1</v>
       </c>
@@ -12375,10 +11019,6 @@
       <c r="H341" t="n">
         <v>2</v>
       </c>
-      <c r="I341" t="inlineStr"/>
-      <c r="J341" t="inlineStr"/>
-      <c r="K341" t="inlineStr"/>
-      <c r="L341" t="inlineStr"/>
       <c r="M341" t="n">
         <v>1</v>
       </c>
@@ -12410,10 +11050,6 @@
       <c r="H342" t="n">
         <v>3</v>
       </c>
-      <c r="I342" t="inlineStr"/>
-      <c r="J342" t="inlineStr"/>
-      <c r="K342" t="inlineStr"/>
-      <c r="L342" t="inlineStr"/>
       <c r="M342" t="n">
         <v>1</v>
       </c>
@@ -12445,10 +11081,6 @@
       <c r="H343" t="n">
         <v>3</v>
       </c>
-      <c r="I343" t="inlineStr"/>
-      <c r="J343" t="inlineStr"/>
-      <c r="K343" t="inlineStr"/>
-      <c r="L343" t="inlineStr"/>
       <c r="M343" t="n">
         <v>1</v>
       </c>
@@ -12480,10 +11112,6 @@
       <c r="H344" t="n">
         <v>1</v>
       </c>
-      <c r="I344" t="inlineStr"/>
-      <c r="J344" t="inlineStr"/>
-      <c r="K344" t="inlineStr"/>
-      <c r="L344" t="inlineStr"/>
       <c r="M344" t="n">
         <v>1</v>
       </c>
@@ -12515,10 +11143,6 @@
       <c r="H345" t="n">
         <v>2</v>
       </c>
-      <c r="I345" t="inlineStr"/>
-      <c r="J345" t="inlineStr"/>
-      <c r="K345" t="inlineStr"/>
-      <c r="L345" t="inlineStr"/>
       <c r="M345" t="n">
         <v>1</v>
       </c>
@@ -12550,10 +11174,6 @@
       <c r="H346" t="n">
         <v>2</v>
       </c>
-      <c r="I346" t="inlineStr"/>
-      <c r="J346" t="inlineStr"/>
-      <c r="K346" t="inlineStr"/>
-      <c r="L346" t="inlineStr"/>
       <c r="M346" t="n">
         <v>1</v>
       </c>
@@ -12585,10 +11205,6 @@
       <c r="H347" t="n">
         <v>2</v>
       </c>
-      <c r="I347" t="inlineStr"/>
-      <c r="J347" t="inlineStr"/>
-      <c r="K347" t="inlineStr"/>
-      <c r="L347" t="inlineStr"/>
       <c r="M347" t="n">
         <v>1</v>
       </c>
@@ -12620,10 +11236,6 @@
       <c r="H348" t="n">
         <v>3</v>
       </c>
-      <c r="I348" t="inlineStr"/>
-      <c r="J348" t="inlineStr"/>
-      <c r="K348" t="inlineStr"/>
-      <c r="L348" t="inlineStr"/>
       <c r="M348" t="n">
         <v>1</v>
       </c>
@@ -12655,10 +11267,6 @@
       <c r="H349" t="n">
         <v>1</v>
       </c>
-      <c r="I349" t="inlineStr"/>
-      <c r="J349" t="inlineStr"/>
-      <c r="K349" t="inlineStr"/>
-      <c r="L349" t="inlineStr"/>
       <c r="M349" t="n">
         <v>1</v>
       </c>
@@ -12690,10 +11298,6 @@
       <c r="H350" t="n">
         <v>3</v>
       </c>
-      <c r="I350" t="inlineStr"/>
-      <c r="J350" t="inlineStr"/>
-      <c r="K350" t="inlineStr"/>
-      <c r="L350" t="inlineStr"/>
       <c r="M350" t="n">
         <v>1</v>
       </c>
@@ -12725,10 +11329,6 @@
       <c r="H351" t="n">
         <v>3</v>
       </c>
-      <c r="I351" t="inlineStr"/>
-      <c r="J351" t="inlineStr"/>
-      <c r="K351" t="inlineStr"/>
-      <c r="L351" t="inlineStr"/>
       <c r="M351" t="n">
         <v>1</v>
       </c>
@@ -12760,10 +11360,6 @@
       <c r="H352" t="n">
         <v>1</v>
       </c>
-      <c r="I352" t="inlineStr"/>
-      <c r="J352" t="inlineStr"/>
-      <c r="K352" t="inlineStr"/>
-      <c r="L352" t="inlineStr"/>
       <c r="M352" t="n">
         <v>1</v>
       </c>
@@ -12795,10 +11391,6 @@
       <c r="H353" t="n">
         <v>2</v>
       </c>
-      <c r="I353" t="inlineStr"/>
-      <c r="J353" t="inlineStr"/>
-      <c r="K353" t="inlineStr"/>
-      <c r="L353" t="inlineStr"/>
       <c r="M353" t="n">
         <v>1</v>
       </c>
@@ -12830,10 +11422,6 @@
       <c r="H354" t="n">
         <v>3</v>
       </c>
-      <c r="I354" t="inlineStr"/>
-      <c r="J354" t="inlineStr"/>
-      <c r="K354" t="inlineStr"/>
-      <c r="L354" t="inlineStr"/>
       <c r="M354" t="n">
         <v>1</v>
       </c>
@@ -12865,10 +11453,6 @@
       <c r="H355" t="n">
         <v>1</v>
       </c>
-      <c r="I355" t="inlineStr"/>
-      <c r="J355" t="inlineStr"/>
-      <c r="K355" t="inlineStr"/>
-      <c r="L355" t="inlineStr"/>
       <c r="M355" t="n">
         <v>1</v>
       </c>
@@ -12900,10 +11484,6 @@
       <c r="H356" t="n">
         <v>2</v>
       </c>
-      <c r="I356" t="inlineStr"/>
-      <c r="J356" t="inlineStr"/>
-      <c r="K356" t="inlineStr"/>
-      <c r="L356" t="inlineStr"/>
       <c r="M356" t="n">
         <v>1</v>
       </c>
@@ -12935,10 +11515,6 @@
       <c r="H357" t="n">
         <v>3</v>
       </c>
-      <c r="I357" t="inlineStr"/>
-      <c r="J357" t="inlineStr"/>
-      <c r="K357" t="inlineStr"/>
-      <c r="L357" t="inlineStr"/>
       <c r="M357" t="n">
         <v>1</v>
       </c>
@@ -12970,10 +11546,6 @@
       <c r="H358" t="n">
         <v>1</v>
       </c>
-      <c r="I358" t="inlineStr"/>
-      <c r="J358" t="inlineStr"/>
-      <c r="K358" t="inlineStr"/>
-      <c r="L358" t="inlineStr"/>
       <c r="M358" t="n">
         <v>1</v>
       </c>
@@ -13005,10 +11577,6 @@
       <c r="H359" t="n">
         <v>2</v>
       </c>
-      <c r="I359" t="inlineStr"/>
-      <c r="J359" t="inlineStr"/>
-      <c r="K359" t="inlineStr"/>
-      <c r="L359" t="inlineStr"/>
       <c r="M359" t="n">
         <v>1</v>
       </c>
@@ -13040,10 +11608,6 @@
       <c r="H360" t="n">
         <v>3</v>
       </c>
-      <c r="I360" t="inlineStr"/>
-      <c r="J360" t="inlineStr"/>
-      <c r="K360" t="inlineStr"/>
-      <c r="L360" t="inlineStr"/>
       <c r="M360" t="n">
         <v>1</v>
       </c>
@@ -13075,10 +11639,6 @@
       <c r="H361" t="n">
         <v>1</v>
       </c>
-      <c r="I361" t="inlineStr"/>
-      <c r="J361" t="inlineStr"/>
-      <c r="K361" t="inlineStr"/>
-      <c r="L361" t="inlineStr"/>
       <c r="M361" t="n">
         <v>1</v>
       </c>
@@ -13110,10 +11670,6 @@
       <c r="H362" t="n">
         <v>2</v>
       </c>
-      <c r="I362" t="inlineStr"/>
-      <c r="J362" t="inlineStr"/>
-      <c r="K362" t="inlineStr"/>
-      <c r="L362" t="inlineStr"/>
       <c r="M362" t="n">
         <v>1</v>
       </c>
@@ -13145,10 +11701,6 @@
       <c r="H363" t="n">
         <v>3</v>
       </c>
-      <c r="I363" t="inlineStr"/>
-      <c r="J363" t="inlineStr"/>
-      <c r="K363" t="inlineStr"/>
-      <c r="L363" t="inlineStr"/>
       <c r="M363" t="n">
         <v>1</v>
       </c>
@@ -13180,10 +11732,6 @@
       <c r="H364" t="n">
         <v>1</v>
       </c>
-      <c r="I364" t="inlineStr"/>
-      <c r="J364" t="inlineStr"/>
-      <c r="K364" t="inlineStr"/>
-      <c r="L364" t="inlineStr"/>
       <c r="M364" t="n">
         <v>1</v>
       </c>
@@ -13215,10 +11763,6 @@
       <c r="H365" t="n">
         <v>2</v>
       </c>
-      <c r="I365" t="inlineStr"/>
-      <c r="J365" t="inlineStr"/>
-      <c r="K365" t="inlineStr"/>
-      <c r="L365" t="inlineStr"/>
       <c r="M365" t="n">
         <v>1</v>
       </c>
@@ -13250,10 +11794,6 @@
       <c r="H366" t="n">
         <v>2</v>
       </c>
-      <c r="I366" t="inlineStr"/>
-      <c r="J366" t="inlineStr"/>
-      <c r="K366" t="inlineStr"/>
-      <c r="L366" t="inlineStr"/>
       <c r="M366" t="n">
         <v>1</v>
       </c>
@@ -13285,10 +11825,6 @@
       <c r="H367" t="n">
         <v>3</v>
       </c>
-      <c r="I367" t="inlineStr"/>
-      <c r="J367" t="inlineStr"/>
-      <c r="K367" t="inlineStr"/>
-      <c r="L367" t="inlineStr"/>
       <c r="M367" t="n">
         <v>1</v>
       </c>
@@ -13320,10 +11856,6 @@
       <c r="H368" t="n">
         <v>1</v>
       </c>
-      <c r="I368" t="inlineStr"/>
-      <c r="J368" t="inlineStr"/>
-      <c r="K368" t="inlineStr"/>
-      <c r="L368" t="inlineStr"/>
       <c r="M368" t="n">
         <v>1</v>
       </c>
@@ -13355,10 +11887,6 @@
       <c r="H369" t="n">
         <v>3</v>
       </c>
-      <c r="I369" t="inlineStr"/>
-      <c r="J369" t="inlineStr"/>
-      <c r="K369" t="inlineStr"/>
-      <c r="L369" t="inlineStr"/>
       <c r="M369" t="n">
         <v>1</v>
       </c>
@@ -13372,7 +11900,7 @@
       </c>
       <c r="C370" t="inlineStr">
         <is>
-          <t>Reconciliation Item</t>
+          <t>Reconciliation of Operating Income (Loss)</t>
         </is>
       </c>
       <c r="D370" t="n">
@@ -13390,10 +11918,6 @@
       <c r="H370" t="n">
         <v>1</v>
       </c>
-      <c r="I370" t="inlineStr"/>
-      <c r="J370" t="inlineStr"/>
-      <c r="K370" t="inlineStr"/>
-      <c r="L370" t="inlineStr"/>
       <c r="M370" t="n">
         <v>1</v>
       </c>
@@ -13425,10 +11949,6 @@
       <c r="H371" t="n">
         <v>2</v>
       </c>
-      <c r="I371" t="inlineStr"/>
-      <c r="J371" t="inlineStr"/>
-      <c r="K371" t="inlineStr"/>
-      <c r="L371" t="inlineStr"/>
       <c r="M371" t="n">
         <v>1</v>
       </c>
@@ -13460,10 +11980,6 @@
       <c r="H372" t="n">
         <v>1</v>
       </c>
-      <c r="I372" t="inlineStr"/>
-      <c r="J372" t="inlineStr"/>
-      <c r="K372" t="inlineStr"/>
-      <c r="L372" t="inlineStr"/>
       <c r="M372" t="n">
         <v>1</v>
       </c>
@@ -13495,10 +12011,6 @@
       <c r="H373" t="n">
         <v>2</v>
       </c>
-      <c r="I373" t="inlineStr"/>
-      <c r="J373" t="inlineStr"/>
-      <c r="K373" t="inlineStr"/>
-      <c r="L373" t="inlineStr"/>
       <c r="M373" t="n">
         <v>1</v>
       </c>
@@ -13530,10 +12042,6 @@
       <c r="H374" t="n">
         <v>1</v>
       </c>
-      <c r="I374" t="inlineStr"/>
-      <c r="J374" t="inlineStr"/>
-      <c r="K374" t="inlineStr"/>
-      <c r="L374" t="inlineStr"/>
       <c r="M374" t="n">
         <v>1</v>
       </c>
@@ -13565,10 +12073,6 @@
       <c r="H375" t="n">
         <v>2</v>
       </c>
-      <c r="I375" t="inlineStr"/>
-      <c r="J375" t="inlineStr"/>
-      <c r="K375" t="inlineStr"/>
-      <c r="L375" t="inlineStr"/>
       <c r="M375" t="n">
         <v>1</v>
       </c>
@@ -13600,10 +12104,6 @@
       <c r="H376" t="n">
         <v>2</v>
       </c>
-      <c r="I376" t="inlineStr"/>
-      <c r="J376" t="inlineStr"/>
-      <c r="K376" t="inlineStr"/>
-      <c r="L376" t="inlineStr"/>
       <c r="M376" t="n">
         <v>1</v>
       </c>
@@ -13635,10 +12135,6 @@
       <c r="H377" t="n">
         <v>2</v>
       </c>
-      <c r="I377" t="inlineStr"/>
-      <c r="J377" t="inlineStr"/>
-      <c r="K377" t="inlineStr"/>
-      <c r="L377" t="inlineStr"/>
       <c r="M377" t="n">
         <v>1</v>
       </c>
@@ -13670,10 +12166,6 @@
       <c r="H378" t="n">
         <v>2</v>
       </c>
-      <c r="I378" t="inlineStr"/>
-      <c r="J378" t="inlineStr"/>
-      <c r="K378" t="inlineStr"/>
-      <c r="L378" t="inlineStr"/>
       <c r="M378" t="n">
         <v>1</v>
       </c>
@@ -13705,10 +12197,6 @@
       <c r="H379" t="n">
         <v>2</v>
       </c>
-      <c r="I379" t="inlineStr"/>
-      <c r="J379" t="inlineStr"/>
-      <c r="K379" t="inlineStr"/>
-      <c r="L379" t="inlineStr"/>
       <c r="M379" t="n">
         <v>1</v>
       </c>
@@ -13740,10 +12228,6 @@
       <c r="H380" t="n">
         <v>2</v>
       </c>
-      <c r="I380" t="inlineStr"/>
-      <c r="J380" t="inlineStr"/>
-      <c r="K380" t="inlineStr"/>
-      <c r="L380" t="inlineStr"/>
       <c r="M380" t="n">
         <v>1</v>
       </c>
@@ -13775,10 +12259,6 @@
       <c r="H381" t="n">
         <v>2</v>
       </c>
-      <c r="I381" t="inlineStr"/>
-      <c r="J381" t="inlineStr"/>
-      <c r="K381" t="inlineStr"/>
-      <c r="L381" t="inlineStr"/>
       <c r="M381" t="n">
         <v>1</v>
       </c>
@@ -13810,10 +12290,6 @@
       <c r="H382" t="n">
         <v>2</v>
       </c>
-      <c r="I382" t="inlineStr"/>
-      <c r="J382" t="inlineStr"/>
-      <c r="K382" t="inlineStr"/>
-      <c r="L382" t="inlineStr"/>
       <c r="M382" t="n">
         <v>1</v>
       </c>
@@ -13845,10 +12321,6 @@
       <c r="H383" t="n">
         <v>3</v>
       </c>
-      <c r="I383" t="inlineStr"/>
-      <c r="J383" t="inlineStr"/>
-      <c r="K383" t="inlineStr"/>
-      <c r="L383" t="inlineStr"/>
       <c r="M383" t="n">
         <v>1</v>
       </c>
@@ -13880,10 +12352,6 @@
       <c r="H384" t="n">
         <v>1</v>
       </c>
-      <c r="I384" t="inlineStr"/>
-      <c r="J384" t="inlineStr"/>
-      <c r="K384" t="inlineStr"/>
-      <c r="L384" t="inlineStr"/>
       <c r="M384" t="n">
         <v>1</v>
       </c>
@@ -13915,10 +12383,6 @@
       <c r="H385" t="n">
         <v>2</v>
       </c>
-      <c r="I385" t="inlineStr"/>
-      <c r="J385" t="inlineStr"/>
-      <c r="K385" t="inlineStr"/>
-      <c r="L385" t="inlineStr"/>
       <c r="M385" t="n">
         <v>1</v>
       </c>
@@ -13950,10 +12414,6 @@
       <c r="H386" t="n">
         <v>2</v>
       </c>
-      <c r="I386" t="inlineStr"/>
-      <c r="J386" t="inlineStr"/>
-      <c r="K386" t="inlineStr"/>
-      <c r="L386" t="inlineStr"/>
       <c r="M386" t="n">
         <v>1</v>
       </c>
@@ -13985,10 +12445,6 @@
       <c r="H387" t="n">
         <v>2</v>
       </c>
-      <c r="I387" t="inlineStr"/>
-      <c r="J387" t="inlineStr"/>
-      <c r="K387" t="inlineStr"/>
-      <c r="L387" t="inlineStr"/>
       <c r="M387" t="n">
         <v>1</v>
       </c>
@@ -14020,10 +12476,6 @@
       <c r="H388" t="n">
         <v>2</v>
       </c>
-      <c r="I388" t="inlineStr"/>
-      <c r="J388" t="inlineStr"/>
-      <c r="K388" t="inlineStr"/>
-      <c r="L388" t="inlineStr"/>
       <c r="M388" t="n">
         <v>1</v>
       </c>
@@ -14055,10 +12507,6 @@
       <c r="H389" t="n">
         <v>2</v>
       </c>
-      <c r="I389" t="inlineStr"/>
-      <c r="J389" t="inlineStr"/>
-      <c r="K389" t="inlineStr"/>
-      <c r="L389" t="inlineStr"/>
       <c r="M389" t="n">
         <v>1</v>
       </c>
@@ -14090,10 +12538,6 @@
       <c r="H390" t="n">
         <v>2</v>
       </c>
-      <c r="I390" t="inlineStr"/>
-      <c r="J390" t="inlineStr"/>
-      <c r="K390" t="inlineStr"/>
-      <c r="L390" t="inlineStr"/>
       <c r="M390" t="n">
         <v>1</v>
       </c>
@@ -14125,10 +12569,6 @@
       <c r="H391" t="n">
         <v>2</v>
       </c>
-      <c r="I391" t="inlineStr"/>
-      <c r="J391" t="inlineStr"/>
-      <c r="K391" t="inlineStr"/>
-      <c r="L391" t="inlineStr"/>
       <c r="M391" t="n">
         <v>1</v>
       </c>
@@ -14160,10 +12600,6 @@
       <c r="H392" t="n">
         <v>2</v>
       </c>
-      <c r="I392" t="inlineStr"/>
-      <c r="J392" t="inlineStr"/>
-      <c r="K392" t="inlineStr"/>
-      <c r="L392" t="inlineStr"/>
       <c r="M392" t="n">
         <v>1</v>
       </c>
@@ -14195,10 +12631,6 @@
       <c r="H393" t="n">
         <v>3</v>
       </c>
-      <c r="I393" t="inlineStr"/>
-      <c r="J393" t="inlineStr"/>
-      <c r="K393" t="inlineStr"/>
-      <c r="L393" t="inlineStr"/>
       <c r="M393" t="n">
         <v>1</v>
       </c>
@@ -14230,10 +12662,6 @@
       <c r="H394" t="n">
         <v>1</v>
       </c>
-      <c r="I394" t="inlineStr"/>
-      <c r="J394" t="inlineStr"/>
-      <c r="K394" t="inlineStr"/>
-      <c r="L394" t="inlineStr"/>
       <c r="M394" t="n">
         <v>1</v>
       </c>
@@ -14265,10 +12693,6 @@
       <c r="H395" t="n">
         <v>2</v>
       </c>
-      <c r="I395" t="inlineStr"/>
-      <c r="J395" t="inlineStr"/>
-      <c r="K395" t="inlineStr"/>
-      <c r="L395" t="inlineStr"/>
       <c r="M395" t="n">
         <v>1</v>
       </c>
@@ -14300,10 +12724,6 @@
       <c r="H396" t="n">
         <v>2</v>
       </c>
-      <c r="I396" t="inlineStr"/>
-      <c r="J396" t="inlineStr"/>
-      <c r="K396" t="inlineStr"/>
-      <c r="L396" t="inlineStr"/>
       <c r="M396" t="n">
         <v>1</v>
       </c>
@@ -14335,10 +12755,6 @@
       <c r="H397" t="n">
         <v>2</v>
       </c>
-      <c r="I397" t="inlineStr"/>
-      <c r="J397" t="inlineStr"/>
-      <c r="K397" t="inlineStr"/>
-      <c r="L397" t="inlineStr"/>
       <c r="M397" t="n">
         <v>1</v>
       </c>
@@ -14370,10 +12786,6 @@
       <c r="H398" t="n">
         <v>2</v>
       </c>
-      <c r="I398" t="inlineStr"/>
-      <c r="J398" t="inlineStr"/>
-      <c r="K398" t="inlineStr"/>
-      <c r="L398" t="inlineStr"/>
       <c r="M398" t="n">
         <v>1</v>
       </c>
@@ -14405,10 +12817,6 @@
       <c r="H399" t="n">
         <v>2</v>
       </c>
-      <c r="I399" t="inlineStr"/>
-      <c r="J399" t="inlineStr"/>
-      <c r="K399" t="inlineStr"/>
-      <c r="L399" t="inlineStr"/>
       <c r="M399" t="n">
         <v>1</v>
       </c>
@@ -14440,10 +12848,6 @@
       <c r="H400" t="n">
         <v>2</v>
       </c>
-      <c r="I400" t="inlineStr"/>
-      <c r="J400" t="inlineStr"/>
-      <c r="K400" t="inlineStr"/>
-      <c r="L400" t="inlineStr"/>
       <c r="M400" t="n">
         <v>1</v>
       </c>
@@ -14475,10 +12879,6 @@
       <c r="H401" t="n">
         <v>2</v>
       </c>
-      <c r="I401" t="inlineStr"/>
-      <c r="J401" t="inlineStr"/>
-      <c r="K401" t="inlineStr"/>
-      <c r="L401" t="inlineStr"/>
       <c r="M401" t="n">
         <v>1</v>
       </c>
@@ -14510,10 +12910,6 @@
       <c r="H402" t="n">
         <v>2</v>
       </c>
-      <c r="I402" t="inlineStr"/>
-      <c r="J402" t="inlineStr"/>
-      <c r="K402" t="inlineStr"/>
-      <c r="L402" t="inlineStr"/>
       <c r="M402" t="n">
         <v>1</v>
       </c>
@@ -14545,10 +12941,6 @@
       <c r="H403" t="n">
         <v>3</v>
       </c>
-      <c r="I403" t="inlineStr"/>
-      <c r="J403" t="inlineStr"/>
-      <c r="K403" t="inlineStr"/>
-      <c r="L403" t="inlineStr"/>
       <c r="M403" t="n">
         <v>1</v>
       </c>
@@ -14580,10 +12972,6 @@
       <c r="H404" t="n">
         <v>1</v>
       </c>
-      <c r="I404" t="inlineStr"/>
-      <c r="J404" t="inlineStr"/>
-      <c r="K404" t="inlineStr"/>
-      <c r="L404" t="inlineStr"/>
       <c r="M404" t="n">
         <v>1</v>
       </c>
@@ -14615,10 +13003,6 @@
       <c r="H405" t="n">
         <v>2</v>
       </c>
-      <c r="I405" t="inlineStr"/>
-      <c r="J405" t="inlineStr"/>
-      <c r="K405" t="inlineStr"/>
-      <c r="L405" t="inlineStr"/>
       <c r="M405" t="n">
         <v>1</v>
       </c>
@@ -14650,10 +13034,6 @@
       <c r="H406" t="n">
         <v>2</v>
       </c>
-      <c r="I406" t="inlineStr"/>
-      <c r="J406" t="inlineStr"/>
-      <c r="K406" t="inlineStr"/>
-      <c r="L406" t="inlineStr"/>
       <c r="M406" t="n">
         <v>1</v>
       </c>
@@ -14685,10 +13065,6 @@
       <c r="H407" t="n">
         <v>2</v>
       </c>
-      <c r="I407" t="inlineStr"/>
-      <c r="J407" t="inlineStr"/>
-      <c r="K407" t="inlineStr"/>
-      <c r="L407" t="inlineStr"/>
       <c r="M407" t="n">
         <v>1</v>
       </c>
@@ -14720,10 +13096,6 @@
       <c r="H408" t="n">
         <v>2</v>
       </c>
-      <c r="I408" t="inlineStr"/>
-      <c r="J408" t="inlineStr"/>
-      <c r="K408" t="inlineStr"/>
-      <c r="L408" t="inlineStr"/>
       <c r="M408" t="n">
         <v>1</v>
       </c>
@@ -14755,10 +13127,6 @@
       <c r="H409" t="n">
         <v>3</v>
       </c>
-      <c r="I409" t="inlineStr"/>
-      <c r="J409" t="inlineStr"/>
-      <c r="K409" t="inlineStr"/>
-      <c r="L409" t="inlineStr"/>
       <c r="M409" t="n">
         <v>1</v>
       </c>
@@ -14790,10 +13158,6 @@
       <c r="H410" t="n">
         <v>3</v>
       </c>
-      <c r="I410" t="inlineStr"/>
-      <c r="J410" t="inlineStr"/>
-      <c r="K410" t="inlineStr"/>
-      <c r="L410" t="inlineStr"/>
       <c r="M410" t="n">
         <v>1</v>
       </c>
@@ -14825,10 +13189,6 @@
       <c r="H411" t="n">
         <v>3</v>
       </c>
-      <c r="I411" t="inlineStr"/>
-      <c r="J411" t="inlineStr"/>
-      <c r="K411" t="inlineStr"/>
-      <c r="L411" t="inlineStr"/>
       <c r="M411" t="n">
         <v>1</v>
       </c>
@@ -14860,10 +13220,6 @@
       <c r="H412" t="n">
         <v>3</v>
       </c>
-      <c r="I412" t="inlineStr"/>
-      <c r="J412" t="inlineStr"/>
-      <c r="K412" t="inlineStr"/>
-      <c r="L412" t="inlineStr"/>
       <c r="M412" t="n">
         <v>1</v>
       </c>
@@ -14895,10 +13251,6 @@
       <c r="H413" t="n">
         <v>1</v>
       </c>
-      <c r="I413" t="inlineStr"/>
-      <c r="J413" t="inlineStr"/>
-      <c r="K413" t="inlineStr"/>
-      <c r="L413" t="inlineStr"/>
       <c r="M413" t="n">
         <v>1</v>
       </c>
@@ -14930,10 +13282,6 @@
       <c r="H414" t="n">
         <v>2</v>
       </c>
-      <c r="I414" t="inlineStr"/>
-      <c r="J414" t="inlineStr"/>
-      <c r="K414" t="inlineStr"/>
-      <c r="L414" t="inlineStr"/>
       <c r="M414" t="n">
         <v>1</v>
       </c>
@@ -14965,10 +13313,6 @@
       <c r="H415" t="n">
         <v>2</v>
       </c>
-      <c r="I415" t="inlineStr"/>
-      <c r="J415" t="inlineStr"/>
-      <c r="K415" t="inlineStr"/>
-      <c r="L415" t="inlineStr"/>
       <c r="M415" t="n">
         <v>1</v>
       </c>
@@ -15000,10 +13344,6 @@
       <c r="H416" t="n">
         <v>2</v>
       </c>
-      <c r="I416" t="inlineStr"/>
-      <c r="J416" t="inlineStr"/>
-      <c r="K416" t="inlineStr"/>
-      <c r="L416" t="inlineStr"/>
       <c r="M416" t="n">
         <v>1</v>
       </c>
@@ -15035,10 +13375,6 @@
       <c r="H417" t="n">
         <v>2</v>
       </c>
-      <c r="I417" t="inlineStr"/>
-      <c r="J417" t="inlineStr"/>
-      <c r="K417" t="inlineStr"/>
-      <c r="L417" t="inlineStr"/>
       <c r="M417" t="n">
         <v>1</v>
       </c>
@@ -15070,10 +13406,6 @@
       <c r="H418" t="n">
         <v>3</v>
       </c>
-      <c r="I418" t="inlineStr"/>
-      <c r="J418" t="inlineStr"/>
-      <c r="K418" t="inlineStr"/>
-      <c r="L418" t="inlineStr"/>
       <c r="M418" t="n">
         <v>1</v>
       </c>
@@ -15105,10 +13437,6 @@
       <c r="H419" t="n">
         <v>3</v>
       </c>
-      <c r="I419" t="inlineStr"/>
-      <c r="J419" t="inlineStr"/>
-      <c r="K419" t="inlineStr"/>
-      <c r="L419" t="inlineStr"/>
       <c r="M419" t="n">
         <v>1</v>
       </c>
@@ -15140,10 +13468,6 @@
       <c r="H420" t="n">
         <v>3</v>
       </c>
-      <c r="I420" t="inlineStr"/>
-      <c r="J420" t="inlineStr"/>
-      <c r="K420" t="inlineStr"/>
-      <c r="L420" t="inlineStr"/>
       <c r="M420" t="n">
         <v>1</v>
       </c>
@@ -15175,10 +13499,6 @@
       <c r="H421" t="n">
         <v>3</v>
       </c>
-      <c r="I421" t="inlineStr"/>
-      <c r="J421" t="inlineStr"/>
-      <c r="K421" t="inlineStr"/>
-      <c r="L421" t="inlineStr"/>
       <c r="M421" t="n">
         <v>1</v>
       </c>
@@ -15210,10 +13530,6 @@
       <c r="H422" t="n">
         <v>1</v>
       </c>
-      <c r="I422" t="inlineStr"/>
-      <c r="J422" t="inlineStr"/>
-      <c r="K422" t="inlineStr"/>
-      <c r="L422" t="inlineStr"/>
       <c r="M422" t="n">
         <v>1</v>
       </c>
@@ -15245,10 +13561,6 @@
       <c r="H423" t="n">
         <v>2</v>
       </c>
-      <c r="I423" t="inlineStr"/>
-      <c r="J423" t="inlineStr"/>
-      <c r="K423" t="inlineStr"/>
-      <c r="L423" t="inlineStr"/>
       <c r="M423" t="n">
         <v>1</v>
       </c>
@@ -15280,10 +13592,6 @@
       <c r="H424" t="n">
         <v>2</v>
       </c>
-      <c r="I424" t="inlineStr"/>
-      <c r="J424" t="inlineStr"/>
-      <c r="K424" t="inlineStr"/>
-      <c r="L424" t="inlineStr"/>
       <c r="M424" t="n">
         <v>1</v>
       </c>
@@ -15315,10 +13623,6 @@
       <c r="H425" t="n">
         <v>2</v>
       </c>
-      <c r="I425" t="inlineStr"/>
-      <c r="J425" t="inlineStr"/>
-      <c r="K425" t="inlineStr"/>
-      <c r="L425" t="inlineStr"/>
       <c r="M425" t="n">
         <v>1</v>
       </c>
@@ -15350,10 +13654,6 @@
       <c r="H426" t="n">
         <v>2</v>
       </c>
-      <c r="I426" t="inlineStr"/>
-      <c r="J426" t="inlineStr"/>
-      <c r="K426" t="inlineStr"/>
-      <c r="L426" t="inlineStr"/>
       <c r="M426" t="n">
         <v>1</v>
       </c>
@@ -15385,10 +13685,6 @@
       <c r="H427" t="n">
         <v>3</v>
       </c>
-      <c r="I427" t="inlineStr"/>
-      <c r="J427" t="inlineStr"/>
-      <c r="K427" t="inlineStr"/>
-      <c r="L427" t="inlineStr"/>
       <c r="M427" t="n">
         <v>1</v>
       </c>
@@ -15420,10 +13716,6 @@
       <c r="H428" t="n">
         <v>3</v>
       </c>
-      <c r="I428" t="inlineStr"/>
-      <c r="J428" t="inlineStr"/>
-      <c r="K428" t="inlineStr"/>
-      <c r="L428" t="inlineStr"/>
       <c r="M428" t="n">
         <v>1</v>
       </c>
@@ -15455,10 +13747,6 @@
       <c r="H429" t="n">
         <v>3</v>
       </c>
-      <c r="I429" t="inlineStr"/>
-      <c r="J429" t="inlineStr"/>
-      <c r="K429" t="inlineStr"/>
-      <c r="L429" t="inlineStr"/>
       <c r="M429" t="n">
         <v>1</v>
       </c>
@@ -15490,10 +13778,6 @@
       <c r="H430" t="n">
         <v>3</v>
       </c>
-      <c r="I430" t="inlineStr"/>
-      <c r="J430" t="inlineStr"/>
-      <c r="K430" t="inlineStr"/>
-      <c r="L430" t="inlineStr"/>
       <c r="M430" t="n">
         <v>1</v>
       </c>
@@ -15525,10 +13809,6 @@
       <c r="H431" t="n">
         <v>1</v>
       </c>
-      <c r="I431" t="inlineStr"/>
-      <c r="J431" t="inlineStr"/>
-      <c r="K431" t="inlineStr"/>
-      <c r="L431" t="inlineStr"/>
       <c r="M431" t="n">
         <v>1</v>
       </c>
@@ -15560,10 +13840,6 @@
       <c r="H432" t="n">
         <v>3</v>
       </c>
-      <c r="I432" t="inlineStr"/>
-      <c r="J432" t="inlineStr"/>
-      <c r="K432" t="inlineStr"/>
-      <c r="L432" t="inlineStr"/>
       <c r="M432" t="n">
         <v>1</v>
       </c>
@@ -15595,10 +13871,6 @@
       <c r="H433" t="n">
         <v>2</v>
       </c>
-      <c r="I433" t="inlineStr"/>
-      <c r="J433" t="inlineStr"/>
-      <c r="K433" t="inlineStr"/>
-      <c r="L433" t="inlineStr"/>
       <c r="M433" t="n">
         <v>1</v>
       </c>
@@ -15630,10 +13902,6 @@
       <c r="H434" t="n">
         <v>3</v>
       </c>
-      <c r="I434" t="inlineStr"/>
-      <c r="J434" t="inlineStr"/>
-      <c r="K434" t="inlineStr"/>
-      <c r="L434" t="inlineStr"/>
       <c r="M434" t="n">
         <v>1</v>
       </c>
@@ -15665,10 +13933,6 @@
       <c r="H435" t="n">
         <v>3</v>
       </c>
-      <c r="I435" t="inlineStr"/>
-      <c r="J435" t="inlineStr"/>
-      <c r="K435" t="inlineStr"/>
-      <c r="L435" t="inlineStr"/>
       <c r="M435" t="n">
         <v>1</v>
       </c>
@@ -15700,10 +13964,6 @@
       <c r="H436" t="n">
         <v>3</v>
       </c>
-      <c r="I436" t="inlineStr"/>
-      <c r="J436" t="inlineStr"/>
-      <c r="K436" t="inlineStr"/>
-      <c r="L436" t="inlineStr"/>
       <c r="M436" t="n">
         <v>1</v>
       </c>
@@ -15735,10 +13995,6 @@
       <c r="H437" t="n">
         <v>3</v>
       </c>
-      <c r="I437" t="inlineStr"/>
-      <c r="J437" t="inlineStr"/>
-      <c r="K437" t="inlineStr"/>
-      <c r="L437" t="inlineStr"/>
       <c r="M437" t="n">
         <v>1</v>
       </c>
@@ -15770,10 +14026,6 @@
       <c r="H438" t="n">
         <v>3</v>
       </c>
-      <c r="I438" t="inlineStr"/>
-      <c r="J438" t="inlineStr"/>
-      <c r="K438" t="inlineStr"/>
-      <c r="L438" t="inlineStr"/>
       <c r="M438" t="n">
         <v>1</v>
       </c>

</xml_diff>